<commit_message>
completed first testbench for decoder
</commit_message>
<xml_diff>
--- a/Resources/InstructionSet.xlsx
+++ b/Resources/InstructionSet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\coding\Nigella\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E68CC0-5D29-40A9-AB9A-17872FB4E4E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F7537A-95FE-4AEE-9041-0E8E5CFD0098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{1780B3F2-89EC-48A1-A04C-A7E74E06A1A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1780B3F2-89EC-48A1-A04C-A7E74E06A1A8}"/>
   </bookViews>
   <sheets>
     <sheet name="OPCODE_encoding" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="209">
   <si>
     <t>N.I.G.E. Machine - instruction set encoding</t>
   </si>
@@ -491,9 +491,6 @@
     <t>Store the character char at memory address addr</t>
   </si>
   <si>
-    <t>?DUP</t>
-  </si>
-  <si>
     <t>x -- 0 | x x</t>
   </si>
   <si>
@@ -581,15 +578,9 @@
     <t>Internal microcode</t>
   </si>
   <si>
-    <t>THROW2</t>
-  </si>
-  <si>
     <t>Second cycle of THROW</t>
   </si>
   <si>
-    <t>REPLACE</t>
-  </si>
-  <si>
     <t>Replace DATA register onto stack</t>
   </si>
   <si>
@@ -651,6 +642,30 @@
   </si>
   <si>
     <t>others =&gt; pf_nxt_1</t>
+  </si>
+  <si>
+    <t>instruction_duration</t>
+  </si>
+  <si>
+    <t>r_stack_op</t>
+  </si>
+  <si>
+    <t>op_nop</t>
+  </si>
+  <si>
+    <t>pf_rts</t>
+  </si>
+  <si>
+    <t>pf_beq</t>
+  </si>
+  <si>
+    <t>pf_bra</t>
+  </si>
+  <si>
+    <t>op_pop</t>
+  </si>
+  <si>
+    <t>op_psh</t>
   </si>
 </sst>
 </file>
@@ -1418,12 +1433,13 @@
     <col min="14" max="14" width="9.5703125" style="2" customWidth="1"/>
     <col min="15" max="15" width="2.7109375" style="6" customWidth="1"/>
     <col min="16" max="16" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="6" customWidth="1"/>
+    <col min="17" max="17" width="18.7109375" style="6" customWidth="1"/>
     <col min="18" max="18" width="9.140625" style="2" customWidth="1"/>
     <col min="19" max="20" width="9.140625" style="2"/>
     <col min="21" max="21" width="3" style="2" customWidth="1"/>
     <col min="22" max="22" width="13.5703125" style="2" customWidth="1"/>
-    <col min="23" max="24" width="3" style="2" customWidth="1"/>
+    <col min="23" max="23" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11" style="2" customWidth="1"/>
     <col min="25" max="25" width="3.5703125" style="2" customWidth="1"/>
     <col min="26" max="26" width="28.85546875" style="7" customWidth="1"/>
     <col min="27" max="27" width="17.7109375" style="2" customWidth="1"/>
@@ -1473,7 +1489,7 @@
       <c r="S3" s="11"/>
       <c r="T3" s="11"/>
       <c r="V3" s="11" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="W3" s="11"/>
       <c r="X3" s="11"/>
@@ -1496,14 +1512,21 @@
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="P4" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
+        <v>189</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="R4" s="4" t="s">
+        <v>202</v>
+      </c>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
       <c r="V4" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="Z4" s="9" t="s">
         <v>12</v>
@@ -1552,22 +1575,34 @@
         <v>1</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>0</v>
+      </c>
+      <c r="R6" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S6" s="14"/>
       <c r="T6" s="14"/>
       <c r="V6" s="2" t="str">
         <f>_xlfn.CONCAT(H6, " =&gt; ", P6, ", ")</f>
         <v xml:space="preserve">0 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W6" s="2" t="str">
+        <f>_xlfn.CONCAT($H6, " =&gt; ", Q6, ", ")</f>
+        <v xml:space="preserve">0 =&gt; 0, </v>
+      </c>
+      <c r="X6" s="2" t="str">
+        <f>_xlfn.CONCAT($H6, " =&gt; ", R6, ", ")</f>
+        <v xml:space="preserve">0 =&gt; op_nop, </v>
+      </c>
       <c r="Z6" s="16" t="str">
-        <f>"1 "&amp;H6&amp;" INSTRUCTION _"&amp;B6</f>
+        <f t="shared" ref="Z6:Z19" si="0">"1 "&amp;H6&amp;" INSTRUCTION _"&amp;B6</f>
         <v>1 0 INSTRUCTION _NOP</v>
       </c>
       <c r="AA6" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B6&amp;CHAR(34)</f>
+        <f t="shared" ref="AA6:AA19" si="1">CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B6&amp;CHAR(34)</f>
         <v>," NOP"</v>
       </c>
     </row>
@@ -1586,15 +1621,15 @@
         <v>1</v>
       </c>
       <c r="H7" s="4">
-        <f t="shared" ref="H7:H19" si="0">F7+E7*64+D7*128</f>
+        <f t="shared" ref="H7:H19" si="2">F7+E7*64+D7*128</f>
         <v>1</v>
       </c>
       <c r="I7" s="3" t="str">
-        <f t="shared" ref="I7:I19" si="1">DEC2BIN(H7,7)</f>
+        <f t="shared" ref="I7:I19" si="3">DEC2BIN(H7,7)</f>
         <v>0000001</v>
       </c>
       <c r="J7" s="3" t="str">
-        <f t="shared" ref="J7:J19" si="2">DEC2HEX(H7)</f>
+        <f t="shared" ref="J7:J19" si="4">DEC2HEX(H7)</f>
         <v>1</v>
       </c>
       <c r="L7" s="5" t="s">
@@ -1607,22 +1642,34 @@
         <v>1</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>0</v>
+      </c>
+      <c r="R7" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S7" s="14"/>
       <c r="T7" s="14"/>
       <c r="V7" s="2" t="str">
-        <f t="shared" ref="V7:V70" si="3">_xlfn.CONCAT(H7, " =&gt; ", P7, ", ")</f>
+        <f t="shared" ref="V7:V70" si="5">_xlfn.CONCAT(H7, " =&gt; ", P7, ", ")</f>
         <v xml:space="preserve">1 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W7" s="2" t="str">
+        <f t="shared" ref="W7:W70" si="6">_xlfn.CONCAT(H7, " =&gt; ", Q7, ", ")</f>
+        <v xml:space="preserve">1 =&gt; 0, </v>
+      </c>
+      <c r="X7" s="2" t="str">
+        <f t="shared" ref="X7:X19" si="7">_xlfn.CONCAT($H7, " =&gt; ", R7, ", ")</f>
+        <v xml:space="preserve">1 =&gt; op_nop, </v>
+      </c>
       <c r="Z7" s="16" t="str">
-        <f>"1 "&amp;H7&amp;" INSTRUCTION _"&amp;B7</f>
+        <f t="shared" si="0"/>
         <v>1 1 INSTRUCTION _DROP</v>
       </c>
       <c r="AA7" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B7&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," DROP"</v>
       </c>
     </row>
@@ -1641,17 +1688,17 @@
         <v>2</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="I8" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0000010</v>
-      </c>
-      <c r="J8" s="3" t="str">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
+      <c r="I8" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0000010</v>
+      </c>
+      <c r="J8" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
       <c r="L8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1662,22 +1709,34 @@
         <v>1</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>0</v>
+      </c>
+      <c r="R8" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="V8" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">2 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W8" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">2 =&gt; 0, </v>
+      </c>
+      <c r="X8" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">2 =&gt; op_nop, </v>
+      </c>
       <c r="Z8" s="16" t="str">
-        <f>"1 "&amp;H8&amp;" INSTRUCTION _"&amp;B8</f>
+        <f t="shared" si="0"/>
         <v>1 2 INSTRUCTION _DUP</v>
       </c>
       <c r="AA8" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B8&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," DUP"</v>
       </c>
     </row>
@@ -1696,17 +1755,17 @@
         <v>3</v>
       </c>
       <c r="H9" s="4">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="I9" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0000011</v>
-      </c>
-      <c r="J9" s="3" t="str">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
+      <c r="I9" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0000011</v>
+      </c>
+      <c r="J9" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
       <c r="L9" s="5" t="s">
         <v>25</v>
       </c>
@@ -1717,22 +1776,34 @@
         <v>1</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>0</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S9" s="14"/>
       <c r="T9" s="14"/>
       <c r="V9" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">3 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W9" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">3 =&gt; 0, </v>
+      </c>
+      <c r="X9" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">3 =&gt; op_nop, </v>
+      </c>
       <c r="Z9" s="16" t="str">
-        <f>"1 "&amp;H9&amp;" INSTRUCTION _"&amp;B9</f>
+        <f t="shared" si="0"/>
         <v>1 3 INSTRUCTION _SWAP</v>
       </c>
       <c r="AA9" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B9&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," SWAP"</v>
       </c>
     </row>
@@ -1751,17 +1822,17 @@
         <v>4</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="I10" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0000100</v>
-      </c>
-      <c r="J10" s="3" t="str">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
+      <c r="I10" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0000100</v>
+      </c>
+      <c r="J10" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
       <c r="L10" s="5" t="s">
         <v>28</v>
       </c>
@@ -1772,22 +1843,34 @@
         <v>1</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q10" s="3">
+        <v>0</v>
+      </c>
+      <c r="R10" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S10" s="14"/>
       <c r="T10" s="14"/>
       <c r="V10" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">4 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W10" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">4 =&gt; 0, </v>
+      </c>
+      <c r="X10" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">4 =&gt; op_nop, </v>
+      </c>
       <c r="Z10" s="16" t="str">
-        <f>"1 "&amp;H10&amp;" INSTRUCTION _"&amp;B10</f>
+        <f t="shared" si="0"/>
         <v>1 4 INSTRUCTION _OVER</v>
       </c>
       <c r="AA10" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B10&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," OVER"</v>
       </c>
     </row>
@@ -1802,21 +1885,21 @@
         <v>0</v>
       </c>
       <c r="F11" s="3">
-        <f t="shared" ref="F11:F19" si="4">F10+1</f>
+        <f t="shared" ref="F11:F19" si="8">F10+1</f>
         <v>5</v>
       </c>
       <c r="H11" s="4">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I11" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0000101</v>
-      </c>
-      <c r="J11" s="3" t="str">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="I11" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0000101</v>
+      </c>
+      <c r="J11" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
       <c r="L11" s="5" t="s">
         <v>31</v>
       </c>
@@ -1827,22 +1910,34 @@
         <v>1</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q11" s="3">
+        <v>0</v>
+      </c>
+      <c r="R11" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S11" s="14"/>
       <c r="T11" s="14"/>
       <c r="V11" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">5 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W11" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">5 =&gt; 0, </v>
+      </c>
+      <c r="X11" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">5 =&gt; op_nop, </v>
+      </c>
       <c r="Z11" s="16" t="str">
-        <f>"1 "&amp;H11&amp;" INSTRUCTION _"&amp;B11</f>
+        <f t="shared" si="0"/>
         <v>1 5 INSTRUCTION _NIP</v>
       </c>
       <c r="AA11" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B11&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," NIP"</v>
       </c>
     </row>
@@ -1857,21 +1952,21 @@
         <v>0</v>
       </c>
       <c r="F12" s="3">
+        <f t="shared" si="8"/>
+        <v>6</v>
+      </c>
+      <c r="H12" s="4">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="I12" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0000110</v>
+      </c>
+      <c r="J12" s="3" t="str">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="H12" s="4">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="I12" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0000110</v>
-      </c>
-      <c r="J12" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
       <c r="L12" s="5" t="s">
         <v>34</v>
       </c>
@@ -1882,22 +1977,34 @@
         <v>1</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>0</v>
+      </c>
+      <c r="R12" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
       <c r="V12" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">6 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W12" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">6 =&gt; 0, </v>
+      </c>
+      <c r="X12" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">6 =&gt; op_nop, </v>
+      </c>
       <c r="Z12" s="16" t="str">
-        <f>"1 "&amp;H12&amp;" INSTRUCTION _"&amp;B12</f>
+        <f t="shared" si="0"/>
         <v>1 6 INSTRUCTION _ROT</v>
       </c>
       <c r="AA12" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B12&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," ROT"</v>
       </c>
     </row>
@@ -1913,20 +2020,20 @@
         <v>0</v>
       </c>
       <c r="F13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I13" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0000111</v>
       </c>
       <c r="J13" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="K13" s="14"/>
@@ -1941,25 +2048,35 @@
       </c>
       <c r="O13" s="15"/>
       <c r="P13" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>0</v>
+      </c>
+      <c r="R13" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S13" s="14"/>
       <c r="T13" s="14"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">7 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
+      <c r="W13" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">7 =&gt; 0, </v>
+      </c>
+      <c r="X13" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">7 =&gt; op_nop, </v>
+      </c>
       <c r="Z13" s="16" t="str">
-        <f>"1 "&amp;H13&amp;" INSTRUCTION _"&amp;B13</f>
+        <f t="shared" si="0"/>
         <v>1 7 INSTRUCTION _&gt;R</v>
       </c>
       <c r="AA13" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B13&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," &gt;R"</v>
       </c>
     </row>
@@ -1974,21 +2091,21 @@
         <v>0</v>
       </c>
       <c r="F14" s="3">
+        <f t="shared" si="8"/>
+        <v>8</v>
+      </c>
+      <c r="H14" s="4">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="I14" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0001000</v>
+      </c>
+      <c r="J14" s="3" t="str">
         <f t="shared" si="4"/>
         <v>8</v>
       </c>
-      <c r="H14" s="4">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="I14" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0001000</v>
-      </c>
-      <c r="J14" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>8</v>
-      </c>
       <c r="L14" s="5" t="s">
         <v>40</v>
       </c>
@@ -1999,22 +2116,34 @@
         <v>1</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>0</v>
+      </c>
+      <c r="R14" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S14" s="14"/>
       <c r="T14" s="14"/>
       <c r="V14" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">8 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W14" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">8 =&gt; 0, </v>
+      </c>
+      <c r="X14" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">8 =&gt; op_nop, </v>
+      </c>
       <c r="Z14" s="16" t="str">
-        <f>"1 "&amp;H14&amp;" INSTRUCTION _"&amp;B14</f>
+        <f t="shared" si="0"/>
         <v>1 8 INSTRUCTION _R@</v>
       </c>
       <c r="AA14" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B14&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," R@"</v>
       </c>
     </row>
@@ -2030,20 +2159,20 @@
         <v>0</v>
       </c>
       <c r="F15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>9</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I15" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0001001</v>
       </c>
       <c r="J15" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="K15" s="14"/>
@@ -2058,25 +2187,35 @@
       </c>
       <c r="O15" s="15"/>
       <c r="P15" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>0</v>
+      </c>
+      <c r="R15" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S15" s="14"/>
       <c r="T15" s="14"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">9 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
+      <c r="W15" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">9 =&gt; 0, </v>
+      </c>
+      <c r="X15" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">9 =&gt; op_nop, </v>
+      </c>
       <c r="Z15" s="16" t="str">
-        <f>"1 "&amp;H15&amp;" INSTRUCTION _"&amp;B15</f>
+        <f t="shared" si="0"/>
         <v>1 9 INSTRUCTION _R&gt;</v>
       </c>
       <c r="AA15" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B15&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," R&gt;"</v>
       </c>
     </row>
@@ -2092,20 +2231,20 @@
         <v>0</v>
       </c>
       <c r="F16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>10</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="I16" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0001010</v>
       </c>
       <c r="J16" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>A</v>
       </c>
       <c r="K16" s="14"/>
@@ -2120,31 +2259,41 @@
       </c>
       <c r="O16" s="15"/>
       <c r="P16" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>0</v>
+      </c>
+      <c r="R16" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S16" s="14"/>
       <c r="T16" s="14"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">10 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
+      <c r="W16" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">10 =&gt; 0, </v>
+      </c>
+      <c r="X16" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">10 =&gt; op_nop, </v>
+      </c>
       <c r="Z16" s="16" t="str">
-        <f>"1 "&amp;H16&amp;" INSTRUCTION _"&amp;B16</f>
+        <f t="shared" si="0"/>
         <v>1 10 INSTRUCTION _PSP@</v>
       </c>
       <c r="AA16" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B16&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," PSP@"</v>
       </c>
     </row>
     <row r="17" spans="1:27" s="17" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B17" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14">
@@ -2154,20 +2303,20 @@
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>11</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="I17" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0001011</v>
       </c>
       <c r="J17" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>B</v>
       </c>
       <c r="K17" s="14"/>
@@ -2182,25 +2331,35 @@
       </c>
       <c r="O17" s="15"/>
       <c r="P17" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q17" s="3">
+        <v>0</v>
+      </c>
+      <c r="R17" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S17" s="14"/>
       <c r="T17" s="14"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">11 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
+      <c r="W17" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">11 =&gt; 0, </v>
+      </c>
+      <c r="X17" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">11 =&gt; op_nop, </v>
+      </c>
       <c r="Z17" s="16" t="str">
-        <f>"1 "&amp;H17&amp;" INSTRUCTION _"&amp;B17</f>
+        <f t="shared" si="0"/>
         <v>1 11 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA17" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B17&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," UNUSED"</v>
       </c>
     </row>
@@ -2215,19 +2374,19 @@
         <v>0</v>
       </c>
       <c r="F18" s="3">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="H18" s="4">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="I18" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0001100</v>
+      </c>
+      <c r="J18" s="3" t="str">
         <f t="shared" si="4"/>
-        <v>12</v>
-      </c>
-      <c r="H18" s="4">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="I18" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0001100</v>
-      </c>
-      <c r="J18" s="3" t="str">
-        <f t="shared" si="2"/>
         <v>C</v>
       </c>
       <c r="L18" s="13" t="s">
@@ -2240,28 +2399,40 @@
         <v>1</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q18" s="3">
+        <v>0</v>
+      </c>
+      <c r="R18" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S18" s="3"/>
       <c r="T18" s="14"/>
       <c r="V18" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">12 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W18" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">12 =&gt; 0, </v>
+      </c>
+      <c r="X18" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">12 =&gt; op_nop, </v>
+      </c>
       <c r="Z18" s="16" t="str">
-        <f>"1 "&amp;H18&amp;" INSTRUCTION _"&amp;B18</f>
+        <f t="shared" si="0"/>
         <v>1 12 INSTRUCTION _RESETSP</v>
       </c>
       <c r="AA18" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B18&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," RESETSP"</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="B19" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D19" s="3">
         <v>0</v>
@@ -2270,19 +2441,19 @@
         <v>0</v>
       </c>
       <c r="F19" s="3">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="H19" s="4">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="I19" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>0001101</v>
+      </c>
+      <c r="J19" s="3" t="str">
         <f t="shared" si="4"/>
-        <v>13</v>
-      </c>
-      <c r="H19" s="4">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="I19" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>0001101</v>
-      </c>
-      <c r="J19" s="3" t="str">
-        <f t="shared" si="2"/>
         <v>D</v>
       </c>
       <c r="L19" s="5" t="s">
@@ -2295,22 +2466,34 @@
         <v>1</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>0</v>
+      </c>
+      <c r="R19" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S19" s="14"/>
       <c r="T19" s="14"/>
       <c r="V19" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">13 =&gt; pf_nxt_1, </v>
       </c>
+      <c r="W19" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">13 =&gt; 0, </v>
+      </c>
+      <c r="X19" s="2" t="str">
+        <f t="shared" si="7"/>
+        <v xml:space="preserve">13 =&gt; op_nop, </v>
+      </c>
       <c r="Z19" s="16" t="str">
-        <f>"1 "&amp;H19&amp;" INSTRUCTION _"&amp;B19</f>
+        <f t="shared" si="0"/>
         <v>1 13 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA19" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B19&amp;CHAR(34)</f>
+        <f t="shared" si="1"/>
         <v>," UNUSED"</v>
       </c>
     </row>
@@ -2343,15 +2526,15 @@
         <v>14</v>
       </c>
       <c r="H22" s="4">
-        <f t="shared" ref="H22:H29" si="5">F22+E22*64+D22*128</f>
+        <f t="shared" ref="H22:H29" si="9">F22+E22*64+D22*128</f>
         <v>14</v>
       </c>
       <c r="I22" s="3" t="str">
-        <f t="shared" ref="I22:I29" si="6">DEC2BIN(H22,7)</f>
+        <f t="shared" ref="I22:I29" si="10">DEC2BIN(H22,7)</f>
         <v>0001110</v>
       </c>
       <c r="J22" s="3" t="str">
-        <f t="shared" ref="J22:J29" si="7">DEC2HEX(H22)</f>
+        <f t="shared" ref="J22:J29" si="11">DEC2HEX(H22)</f>
         <v>E</v>
       </c>
       <c r="L22" s="5" t="s">
@@ -2364,25 +2547,35 @@
         <v>1</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>0</v>
+      </c>
+      <c r="R22" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S22" s="14"/>
       <c r="T22" s="14"/>
       <c r="U22" s="21"/>
       <c r="V22" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">14 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W22" s="21"/>
-      <c r="X22" s="21"/>
+      <c r="W22" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">14 =&gt; 0, </v>
+      </c>
+      <c r="X22" s="2" t="str">
+        <f t="shared" ref="X22:X29" si="12">_xlfn.CONCAT($H22, " =&gt; ", R22, ", ")</f>
+        <v xml:space="preserve">14 =&gt; op_nop, </v>
+      </c>
       <c r="Z22" s="16" t="str">
-        <f>"1 "&amp;H22&amp;" INSTRUCTION _"&amp;B22</f>
+        <f t="shared" ref="Z22:Z29" si="13">"1 "&amp;H22&amp;" INSTRUCTION _"&amp;B22</f>
         <v>1 14 INSTRUCTION _+</v>
       </c>
       <c r="AA22" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B22&amp;CHAR(34)</f>
+        <f t="shared" ref="AA22:AA29" si="14">CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B22&amp;CHAR(34)</f>
         <v>," +"</v>
       </c>
     </row>
@@ -2402,15 +2595,15 @@
         <v>15</v>
       </c>
       <c r="H23" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>15</v>
       </c>
       <c r="I23" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0001111</v>
       </c>
       <c r="J23" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>F</v>
       </c>
       <c r="L23" s="5" t="s">
@@ -2423,25 +2616,35 @@
         <v>1</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>0</v>
+      </c>
+      <c r="R23" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S23" s="14"/>
       <c r="T23" s="14"/>
       <c r="U23" s="21"/>
       <c r="V23" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">15 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W23" s="21"/>
-      <c r="X23" s="21"/>
+      <c r="W23" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">15 =&gt; 0, </v>
+      </c>
+      <c r="X23" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">15 =&gt; op_nop, </v>
+      </c>
       <c r="Z23" s="16" t="str">
-        <f>"1 "&amp;H23&amp;" INSTRUCTION _"&amp;B23</f>
+        <f t="shared" si="13"/>
         <v>1 15 INSTRUCTION _-</v>
       </c>
       <c r="AA23" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B23&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," -"</v>
       </c>
     </row>
@@ -2456,19 +2659,19 @@
         <v>0</v>
       </c>
       <c r="F24" s="3">
-        <f t="shared" ref="F24:F29" si="8">F23+1</f>
+        <f t="shared" ref="F24:F29" si="15">F23+1</f>
         <v>16</v>
       </c>
       <c r="H24" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>16</v>
       </c>
       <c r="I24" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010000</v>
       </c>
       <c r="J24" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
       <c r="L24" s="5" t="s">
@@ -2481,25 +2684,35 @@
         <v>1</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q24" s="3"/>
-      <c r="R24" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q24" s="3">
+        <v>0</v>
+      </c>
+      <c r="R24" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S24" s="14"/>
       <c r="T24" s="14"/>
       <c r="U24" s="21"/>
       <c r="V24" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">16 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W24" s="21"/>
-      <c r="X24" s="21"/>
+      <c r="W24" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">16 =&gt; 0, </v>
+      </c>
+      <c r="X24" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">16 =&gt; op_nop, </v>
+      </c>
       <c r="Z24" s="16" t="str">
-        <f>"1 "&amp;H24&amp;" INSTRUCTION _"&amp;B24</f>
+        <f t="shared" si="13"/>
         <v>1 16 INSTRUCTION _NEGATE</v>
       </c>
       <c r="AA24" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B24&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," NEGATE"</v>
       </c>
     </row>
@@ -2515,20 +2728,20 @@
         <v>0</v>
       </c>
       <c r="F25" s="3">
-        <f t="shared" si="8"/>
+        <f t="shared" si="15"/>
         <v>17</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>17</v>
       </c>
       <c r="I25" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010001</v>
       </c>
       <c r="J25" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="K25" s="3"/>
@@ -2543,25 +2756,35 @@
       </c>
       <c r="O25" s="15"/>
       <c r="P25" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q25" s="3">
+        <v>0</v>
+      </c>
+      <c r="R25" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S25" s="14"/>
       <c r="T25" s="14"/>
       <c r="U25" s="21"/>
       <c r="V25" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">17 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W25" s="21"/>
-      <c r="X25" s="21"/>
+      <c r="W25" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">17 =&gt; 0, </v>
+      </c>
+      <c r="X25" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">17 =&gt; op_nop, </v>
+      </c>
       <c r="Z25" s="16" t="str">
-        <f>"1 "&amp;H25&amp;" INSTRUCTION _"&amp;B25</f>
+        <f t="shared" si="13"/>
         <v>1 17 INSTRUCTION _1+</v>
       </c>
       <c r="AA25" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B25&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," 1+"</v>
       </c>
     </row>
@@ -2577,20 +2800,20 @@
         <v>0</v>
       </c>
       <c r="F26" s="3">
-        <f t="shared" si="8"/>
+        <f t="shared" si="15"/>
         <v>18</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>18</v>
       </c>
       <c r="I26" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010010</v>
       </c>
       <c r="J26" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>12</v>
       </c>
       <c r="K26" s="3"/>
@@ -2605,25 +2828,35 @@
       </c>
       <c r="O26" s="15"/>
       <c r="P26" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q26" s="3">
+        <v>0</v>
+      </c>
+      <c r="R26" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S26" s="14"/>
       <c r="T26" s="14"/>
       <c r="U26" s="21"/>
       <c r="V26" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">18 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W26" s="21"/>
-      <c r="X26" s="21"/>
+      <c r="W26" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">18 =&gt; 0, </v>
+      </c>
+      <c r="X26" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">18 =&gt; op_nop, </v>
+      </c>
       <c r="Z26" s="16" t="str">
-        <f>"1 "&amp;H26&amp;" INSTRUCTION _"&amp;B26</f>
+        <f t="shared" si="13"/>
         <v>1 18 INSTRUCTION _1-</v>
       </c>
       <c r="AA26" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B26&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," 1-"</v>
       </c>
     </row>
@@ -2644,15 +2877,15 @@
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>19</v>
       </c>
       <c r="I27" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010011</v>
       </c>
       <c r="J27" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>13</v>
       </c>
       <c r="K27" s="3"/>
@@ -2667,25 +2900,35 @@
       </c>
       <c r="O27" s="15"/>
       <c r="P27" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>0</v>
+      </c>
+      <c r="R27" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S27" s="14"/>
       <c r="T27" s="14"/>
       <c r="U27" s="21"/>
       <c r="V27" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">19 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W27" s="21"/>
-      <c r="X27" s="21"/>
+      <c r="W27" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">19 =&gt; 0, </v>
+      </c>
+      <c r="X27" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">19 =&gt; op_nop, </v>
+      </c>
       <c r="Z27" s="16" t="str">
-        <f>"1 "&amp;H27&amp;" INSTRUCTION _"&amp;B27</f>
+        <f t="shared" si="13"/>
         <v>1 19 INSTRUCTION _2/</v>
       </c>
       <c r="AA27" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B27&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," 2/"</v>
       </c>
     </row>
@@ -2706,15 +2949,15 @@
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>20</v>
       </c>
       <c r="I28" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010100</v>
       </c>
       <c r="J28" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>14</v>
       </c>
       <c r="K28" s="14"/>
@@ -2729,25 +2972,35 @@
       </c>
       <c r="O28" s="15"/>
       <c r="P28" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>0</v>
+      </c>
+      <c r="R28" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S28" s="14"/>
       <c r="T28" s="14"/>
       <c r="U28" s="21"/>
       <c r="V28" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">20 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W28" s="21"/>
-      <c r="X28" s="21"/>
+      <c r="W28" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">20 =&gt; 0, </v>
+      </c>
+      <c r="X28" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">20 =&gt; op_nop, </v>
+      </c>
       <c r="Z28" s="16" t="str">
-        <f>"1 "&amp;H28&amp;" INSTRUCTION _"&amp;B28</f>
+        <f t="shared" si="13"/>
         <v>1 20 INSTRUCTION _ADDX</v>
       </c>
       <c r="AA28" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B28&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," ADDX"</v>
       </c>
     </row>
@@ -2763,20 +3016,20 @@
         <v>0</v>
       </c>
       <c r="F29" s="3">
-        <f t="shared" si="8"/>
+        <f t="shared" si="15"/>
         <v>21</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>21</v>
       </c>
       <c r="I29" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0010101</v>
       </c>
       <c r="J29" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>15</v>
       </c>
       <c r="K29" s="14"/>
@@ -2791,25 +3044,35 @@
       </c>
       <c r="O29" s="15"/>
       <c r="P29" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>0</v>
+      </c>
+      <c r="R29" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S29" s="14"/>
       <c r="T29" s="14"/>
       <c r="U29" s="21"/>
       <c r="V29" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">21 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W29" s="21"/>
-      <c r="X29" s="21"/>
+      <c r="W29" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">21 =&gt; 0, </v>
+      </c>
+      <c r="X29" s="2" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">21 =&gt; op_nop, </v>
+      </c>
       <c r="Z29" s="16" t="str">
-        <f>"1 "&amp;H29&amp;" INSTRUCTION _"&amp;B29</f>
+        <f t="shared" si="13"/>
         <v>1 21 INSTRUCTION _SUBX</v>
       </c>
       <c r="AA29" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B29&amp;CHAR(34)</f>
+        <f t="shared" si="14"/>
         <v>," SUBX"</v>
       </c>
     </row>
@@ -2846,15 +3109,15 @@
         <v>22</v>
       </c>
       <c r="H32" s="4">
-        <f t="shared" ref="H32:H42" si="9">F32+E32*64+D32*128</f>
+        <f t="shared" ref="H32:H42" si="16">F32+E32*64+D32*128</f>
         <v>22</v>
       </c>
       <c r="I32" s="3" t="str">
-        <f t="shared" ref="I32:I42" si="10">DEC2BIN(H32,7)</f>
+        <f t="shared" ref="I32:I42" si="17">DEC2BIN(H32,7)</f>
         <v>0010110</v>
       </c>
       <c r="J32" s="3" t="str">
-        <f t="shared" ref="J32:J42" si="11">DEC2HEX(H32)</f>
+        <f t="shared" ref="J32:J42" si="18">DEC2HEX(H32)</f>
         <v>16</v>
       </c>
       <c r="L32" s="5" t="s">
@@ -2867,25 +3130,35 @@
         <v>1</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q32" s="3"/>
-      <c r="R32" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q32" s="3">
+        <v>0</v>
+      </c>
+      <c r="R32" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S32" s="14"/>
       <c r="T32" s="14"/>
       <c r="U32" s="21"/>
       <c r="V32" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">22 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W32" s="21"/>
-      <c r="X32" s="21"/>
+      <c r="W32" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">22 =&gt; 0, </v>
+      </c>
+      <c r="X32" s="2" t="str">
+        <f t="shared" ref="X32:X42" si="19">_xlfn.CONCAT($H32, " =&gt; ", R32, ", ")</f>
+        <v xml:space="preserve">22 =&gt; op_nop, </v>
+      </c>
       <c r="Z32" s="16" t="str">
-        <f>"1 "&amp;H32&amp;" INSTRUCTION _"&amp;B32</f>
+        <f t="shared" ref="Z32:Z42" si="20">"1 "&amp;H32&amp;" INSTRUCTION _"&amp;B32</f>
         <v>1 22 INSTRUCTION _=</v>
       </c>
       <c r="AA32" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B32&amp;CHAR(34)</f>
+        <f t="shared" ref="AA32:AA42" si="21">CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B32&amp;CHAR(34)</f>
         <v>," ="</v>
       </c>
     </row>
@@ -2907,15 +3180,15 @@
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>23</v>
       </c>
       <c r="I33" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0010111</v>
       </c>
       <c r="J33" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>17</v>
       </c>
       <c r="K33" s="14"/>
@@ -2930,25 +3203,35 @@
       </c>
       <c r="O33" s="15"/>
       <c r="P33" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q33" s="3"/>
-      <c r="R33" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q33" s="3">
+        <v>0</v>
+      </c>
+      <c r="R33" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S33" s="14"/>
       <c r="T33" s="14"/>
       <c r="U33" s="21"/>
       <c r="V33" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">23 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W33" s="21"/>
-      <c r="X33" s="21"/>
+      <c r="W33" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">23 =&gt; 0, </v>
+      </c>
+      <c r="X33" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">23 =&gt; op_nop, </v>
+      </c>
       <c r="Z33" s="16" t="str">
-        <f>"1 "&amp;H33&amp;" INSTRUCTION _"&amp;B33</f>
+        <f t="shared" si="20"/>
         <v>1 23 INSTRUCTION _&lt;&gt;</v>
       </c>
       <c r="AA33" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B33&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," &lt;&gt;"</v>
       </c>
     </row>
@@ -2964,20 +3247,20 @@
         <v>0</v>
       </c>
       <c r="F34" s="14">
-        <f t="shared" ref="F34:F42" si="12">F33+1</f>
+        <f t="shared" ref="F34:F42" si="22">F33+1</f>
         <v>24</v>
       </c>
       <c r="G34" s="14"/>
       <c r="H34" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>24</v>
       </c>
       <c r="I34" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011000</v>
       </c>
       <c r="J34" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>18</v>
       </c>
       <c r="L34" s="5" t="s">
@@ -2990,25 +3273,35 @@
         <v>1</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q34" s="3"/>
-      <c r="R34" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>0</v>
+      </c>
+      <c r="R34" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S34" s="14"/>
       <c r="T34" s="14"/>
       <c r="U34" s="21"/>
       <c r="V34" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">24 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W34" s="21"/>
-      <c r="X34" s="21"/>
+      <c r="W34" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">24 =&gt; 0, </v>
+      </c>
+      <c r="X34" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">24 =&gt; op_nop, </v>
+      </c>
       <c r="Z34" s="16" t="str">
-        <f>"1 "&amp;H34&amp;" INSTRUCTION _"&amp;B34</f>
+        <f t="shared" si="20"/>
         <v>1 24 INSTRUCTION _&lt;</v>
       </c>
       <c r="AA34" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B34&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," &lt;"</v>
       </c>
     </row>
@@ -3024,20 +3317,20 @@
         <v>0</v>
       </c>
       <c r="F35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>25</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>25</v>
       </c>
       <c r="I35" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011001</v>
       </c>
       <c r="J35" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>19</v>
       </c>
       <c r="L35" s="5" t="s">
@@ -3050,25 +3343,35 @@
         <v>1</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q35" s="3"/>
-      <c r="R35" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>0</v>
+      </c>
+      <c r="R35" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S35" s="14"/>
       <c r="T35" s="14"/>
       <c r="U35" s="21"/>
       <c r="V35" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">25 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W35" s="21"/>
-      <c r="X35" s="21"/>
+      <c r="W35" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">25 =&gt; 0, </v>
+      </c>
+      <c r="X35" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">25 =&gt; op_nop, </v>
+      </c>
       <c r="Z35" s="16" t="str">
-        <f>"1 "&amp;H35&amp;" INSTRUCTION _"&amp;B35</f>
+        <f t="shared" si="20"/>
         <v>1 25 INSTRUCTION _&gt;</v>
       </c>
       <c r="AA35" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B35&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," &gt;"</v>
       </c>
     </row>
@@ -3084,20 +3387,20 @@
         <v>0</v>
       </c>
       <c r="F36" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>26</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>26</v>
       </c>
       <c r="I36" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011010</v>
       </c>
       <c r="J36" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1A</v>
       </c>
       <c r="L36" s="5" t="s">
@@ -3110,25 +3413,35 @@
         <v>1</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q36" s="3"/>
-      <c r="R36" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>0</v>
+      </c>
+      <c r="R36" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S36" s="14"/>
       <c r="T36" s="14"/>
       <c r="U36" s="21"/>
       <c r="V36" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">26 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W36" s="21"/>
-      <c r="X36" s="21"/>
+      <c r="W36" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">26 =&gt; 0, </v>
+      </c>
+      <c r="X36" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">26 =&gt; op_nop, </v>
+      </c>
       <c r="Z36" s="16" t="str">
-        <f>"1 "&amp;H36&amp;" INSTRUCTION _"&amp;B36</f>
+        <f t="shared" si="20"/>
         <v>1 26 INSTRUCTION _U&lt;</v>
       </c>
       <c r="AA36" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B36&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," U&lt;"</v>
       </c>
     </row>
@@ -3144,20 +3457,20 @@
         <v>0</v>
       </c>
       <c r="F37" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>27</v>
       </c>
       <c r="G37" s="14"/>
       <c r="H37" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>27</v>
       </c>
       <c r="I37" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011011</v>
       </c>
       <c r="J37" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1B</v>
       </c>
       <c r="L37" s="5" t="s">
@@ -3170,25 +3483,35 @@
         <v>1</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q37" s="3"/>
-      <c r="R37" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>0</v>
+      </c>
+      <c r="R37" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S37" s="14"/>
       <c r="T37" s="14"/>
       <c r="U37" s="21"/>
       <c r="V37" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">27 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W37" s="21"/>
-      <c r="X37" s="21"/>
+      <c r="W37" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">27 =&gt; 0, </v>
+      </c>
+      <c r="X37" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">27 =&gt; op_nop, </v>
+      </c>
       <c r="Z37" s="16" t="str">
-        <f>"1 "&amp;H37&amp;" INSTRUCTION _"&amp;B37</f>
+        <f t="shared" si="20"/>
         <v>1 27 INSTRUCTION _U&gt;</v>
       </c>
       <c r="AA37" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B37&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," U&gt;"</v>
       </c>
     </row>
@@ -3205,20 +3528,20 @@
         <v>0</v>
       </c>
       <c r="F38" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>28</v>
       </c>
       <c r="G38" s="14"/>
       <c r="H38" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>28</v>
       </c>
       <c r="I38" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011100</v>
       </c>
       <c r="J38" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1C</v>
       </c>
       <c r="K38" s="14"/>
@@ -3233,25 +3556,35 @@
       </c>
       <c r="O38" s="15"/>
       <c r="P38" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q38" s="3"/>
-      <c r="R38" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>0</v>
+      </c>
+      <c r="R38" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S38" s="14"/>
       <c r="T38" s="14"/>
       <c r="U38" s="21"/>
       <c r="V38" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">28 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W38" s="21"/>
-      <c r="X38" s="21"/>
+      <c r="W38" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">28 =&gt; 0, </v>
+      </c>
+      <c r="X38" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">28 =&gt; op_nop, </v>
+      </c>
       <c r="Z38" s="16" t="str">
-        <f>"1 "&amp;H38&amp;" INSTRUCTION _"&amp;B38</f>
+        <f t="shared" si="20"/>
         <v>1 28 INSTRUCTION _0=</v>
       </c>
       <c r="AA38" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B38&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," 0="</v>
       </c>
     </row>
@@ -3268,20 +3601,20 @@
         <v>0</v>
       </c>
       <c r="F39" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>29</v>
       </c>
       <c r="G39" s="14"/>
       <c r="H39" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>29</v>
       </c>
       <c r="I39" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011101</v>
       </c>
       <c r="J39" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1D</v>
       </c>
       <c r="K39" s="14"/>
@@ -3296,25 +3629,35 @@
       </c>
       <c r="O39" s="15"/>
       <c r="P39" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q39" s="3"/>
-      <c r="R39" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>0</v>
+      </c>
+      <c r="R39" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S39" s="14"/>
       <c r="T39" s="14"/>
       <c r="U39" s="21"/>
       <c r="V39" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">29 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W39" s="21"/>
-      <c r="X39" s="21"/>
+      <c r="W39" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">29 =&gt; 0, </v>
+      </c>
+      <c r="X39" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">29 =&gt; op_nop, </v>
+      </c>
       <c r="Z39" s="16" t="str">
-        <f>"1 "&amp;H39&amp;" INSTRUCTION _"&amp;B39</f>
+        <f t="shared" si="20"/>
         <v>1 29 INSTRUCTION _0&lt;&gt;</v>
       </c>
       <c r="AA39" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B39&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," 0&lt;&gt;"</v>
       </c>
     </row>
@@ -3331,20 +3674,20 @@
         <v>0</v>
       </c>
       <c r="F40" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>30</v>
       </c>
       <c r="G40" s="14"/>
       <c r="H40" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>30</v>
       </c>
       <c r="I40" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011110</v>
       </c>
       <c r="J40" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1E</v>
       </c>
       <c r="K40" s="14"/>
@@ -3359,25 +3702,35 @@
       </c>
       <c r="O40" s="15"/>
       <c r="P40" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q40" s="3"/>
-      <c r="R40" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>0</v>
+      </c>
+      <c r="R40" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S40" s="14"/>
       <c r="T40" s="14"/>
       <c r="U40" s="21"/>
       <c r="V40" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">30 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W40" s="21"/>
-      <c r="X40" s="21"/>
+      <c r="W40" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">30 =&gt; 0, </v>
+      </c>
+      <c r="X40" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">30 =&gt; op_nop, </v>
+      </c>
       <c r="Z40" s="16" t="str">
-        <f>"1 "&amp;H40&amp;" INSTRUCTION _"&amp;B40</f>
+        <f t="shared" si="20"/>
         <v>1 30 INSTRUCTION _0&lt;</v>
       </c>
       <c r="AA40" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B40&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," 0&lt;"</v>
       </c>
     </row>
@@ -3394,20 +3747,20 @@
         <v>0</v>
       </c>
       <c r="F41" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>31</v>
       </c>
       <c r="G41" s="14"/>
       <c r="H41" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>31</v>
       </c>
       <c r="I41" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0011111</v>
       </c>
       <c r="J41" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>1F</v>
       </c>
       <c r="K41" s="14"/>
@@ -3422,25 +3775,35 @@
       </c>
       <c r="O41" s="15"/>
       <c r="P41" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q41" s="3"/>
-      <c r="R41" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>0</v>
+      </c>
+      <c r="R41" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S41" s="14"/>
       <c r="T41" s="14"/>
       <c r="U41" s="21"/>
       <c r="V41" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">31 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W41" s="21"/>
-      <c r="X41" s="21"/>
+      <c r="W41" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">31 =&gt; 0, </v>
+      </c>
+      <c r="X41" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">31 =&gt; op_nop, </v>
+      </c>
       <c r="Z41" s="16" t="str">
-        <f>"1 "&amp;H41&amp;" INSTRUCTION _"&amp;B41</f>
+        <f t="shared" si="20"/>
         <v>1 31 INSTRUCTION _0&gt;</v>
       </c>
       <c r="AA41" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B41&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," 0&gt;"</v>
       </c>
     </row>
@@ -3457,20 +3820,20 @@
         <v>0</v>
       </c>
       <c r="F42" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>32</v>
       </c>
       <c r="G42" s="14"/>
       <c r="H42" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v>32</v>
       </c>
       <c r="I42" s="3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v>0100000</v>
       </c>
       <c r="J42" s="3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>20</v>
       </c>
       <c r="K42" s="14"/>
@@ -3485,25 +3848,35 @@
       </c>
       <c r="O42" s="15"/>
       <c r="P42" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q42" s="3"/>
-      <c r="R42" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q42" s="3">
+        <v>0</v>
+      </c>
+      <c r="R42" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S42" s="14"/>
       <c r="T42" s="14"/>
       <c r="U42" s="21"/>
       <c r="V42" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">32 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W42" s="21"/>
-      <c r="X42" s="21"/>
+      <c r="W42" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">32 =&gt; 0, </v>
+      </c>
+      <c r="X42" s="2" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">32 =&gt; op_nop, </v>
+      </c>
       <c r="Z42" s="16" t="str">
-        <f>"1 "&amp;H42&amp;" INSTRUCTION _"&amp;B42</f>
+        <f t="shared" si="20"/>
         <v>1 32 INSTRUCTION _ZERO</v>
       </c>
       <c r="AA42" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B42&amp;CHAR(34)</f>
+        <f t="shared" si="21"/>
         <v>," ZERO"</v>
       </c>
     </row>
@@ -3538,15 +3911,15 @@
         <v>33</v>
       </c>
       <c r="H45" s="4">
-        <f t="shared" ref="H45:H52" si="13">F45+E45*64+D45*128</f>
+        <f t="shared" ref="H45:H52" si="23">F45+E45*64+D45*128</f>
         <v>33</v>
       </c>
       <c r="I45" s="3" t="str">
-        <f t="shared" ref="I45:I52" si="14">DEC2BIN(H45,7)</f>
+        <f t="shared" ref="I45:I52" si="24">DEC2BIN(H45,7)</f>
         <v>0100001</v>
       </c>
       <c r="J45" s="3" t="str">
-        <f t="shared" ref="J45:J52" si="15">DEC2HEX(H45)</f>
+        <f t="shared" ref="J45:J52" si="25">DEC2HEX(H45)</f>
         <v>21</v>
       </c>
       <c r="L45" s="5" t="s">
@@ -3559,25 +3932,35 @@
         <v>1</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q45" s="3"/>
-      <c r="R45" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q45" s="3">
+        <v>0</v>
+      </c>
+      <c r="R45" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S45" s="14"/>
       <c r="T45" s="14"/>
       <c r="U45" s="21"/>
       <c r="V45" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">33 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W45" s="21"/>
-      <c r="X45" s="21"/>
+      <c r="W45" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">33 =&gt; 0, </v>
+      </c>
+      <c r="X45" s="2" t="str">
+        <f t="shared" ref="X45:X52" si="26">_xlfn.CONCAT($H45, " =&gt; ", R45, ", ")</f>
+        <v xml:space="preserve">33 =&gt; op_nop, </v>
+      </c>
       <c r="Z45" s="16" t="str">
-        <f>"1 "&amp;H45&amp;" INSTRUCTION _"&amp;B45</f>
+        <f t="shared" ref="Z45:Z52" si="27">"1 "&amp;H45&amp;" INSTRUCTION _"&amp;B45</f>
         <v>1 33 INSTRUCTION _AND</v>
       </c>
       <c r="AA45" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B45&amp;CHAR(34)</f>
+        <f t="shared" ref="AA45:AA52" si="28">CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B45&amp;CHAR(34)</f>
         <v>," AND"</v>
       </c>
     </row>
@@ -3597,15 +3980,15 @@
         <v>34</v>
       </c>
       <c r="H46" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>34</v>
       </c>
       <c r="I46" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100010</v>
       </c>
       <c r="J46" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>22</v>
       </c>
       <c r="L46" s="5" t="s">
@@ -3618,25 +4001,35 @@
         <v>1</v>
       </c>
       <c r="P46" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q46" s="3"/>
-      <c r="R46" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q46" s="3">
+        <v>0</v>
+      </c>
+      <c r="R46" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S46" s="14"/>
       <c r="T46" s="14"/>
       <c r="U46" s="21"/>
       <c r="V46" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">34 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W46" s="21"/>
-      <c r="X46" s="21"/>
+      <c r="W46" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">34 =&gt; 0, </v>
+      </c>
+      <c r="X46" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">34 =&gt; op_nop, </v>
+      </c>
       <c r="Z46" s="16" t="str">
-        <f>"1 "&amp;H46&amp;" INSTRUCTION _"&amp;B46</f>
+        <f t="shared" si="27"/>
         <v>1 34 INSTRUCTION _OR</v>
       </c>
       <c r="AA46" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B46&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," OR"</v>
       </c>
     </row>
@@ -3652,19 +4045,19 @@
         <v>0</v>
       </c>
       <c r="F47" s="3">
-        <f t="shared" ref="F47:F52" si="16">F46+1</f>
+        <f t="shared" ref="F47:F52" si="29">F46+1</f>
         <v>35</v>
       </c>
       <c r="H47" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>35</v>
       </c>
       <c r="I47" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100011</v>
       </c>
       <c r="J47" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>23</v>
       </c>
       <c r="L47" s="5" t="s">
@@ -3677,25 +4070,35 @@
         <v>1</v>
       </c>
       <c r="P47" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q47" s="3"/>
-      <c r="R47" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q47" s="3">
+        <v>0</v>
+      </c>
+      <c r="R47" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S47" s="14"/>
       <c r="T47" s="14"/>
       <c r="U47" s="21"/>
       <c r="V47" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">35 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W47" s="21"/>
-      <c r="X47" s="21"/>
+      <c r="W47" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">35 =&gt; 0, </v>
+      </c>
+      <c r="X47" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">35 =&gt; op_nop, </v>
+      </c>
       <c r="Z47" s="16" t="str">
-        <f>"1 "&amp;H47&amp;" INSTRUCTION _"&amp;B47</f>
+        <f t="shared" si="27"/>
         <v>1 35 INSTRUCTION _INVERT</v>
       </c>
       <c r="AA47" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B47&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," INVERT"</v>
       </c>
     </row>
@@ -3711,19 +4114,19 @@
         <v>0</v>
       </c>
       <c r="F48" s="3">
-        <f t="shared" si="16"/>
+        <f t="shared" si="29"/>
         <v>36</v>
       </c>
       <c r="H48" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>36</v>
       </c>
       <c r="I48" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100100</v>
       </c>
       <c r="J48" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>24</v>
       </c>
       <c r="L48" s="5" t="s">
@@ -3736,25 +4139,35 @@
         <v>1</v>
       </c>
       <c r="P48" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q48" s="3"/>
-      <c r="R48" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q48" s="3">
+        <v>0</v>
+      </c>
+      <c r="R48" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S48" s="14"/>
       <c r="T48" s="14"/>
       <c r="U48" s="21"/>
       <c r="V48" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">36 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W48" s="21"/>
-      <c r="X48" s="21"/>
+      <c r="W48" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">36 =&gt; 0, </v>
+      </c>
+      <c r="X48" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">36 =&gt; op_nop, </v>
+      </c>
       <c r="Z48" s="16" t="str">
-        <f>"1 "&amp;H48&amp;" INSTRUCTION _"&amp;B48</f>
+        <f t="shared" si="27"/>
         <v>1 36 INSTRUCTION _XOR</v>
       </c>
       <c r="AA48" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B48&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," XOR"</v>
       </c>
     </row>
@@ -3770,19 +4183,19 @@
         <v>0</v>
       </c>
       <c r="F49" s="3">
-        <f t="shared" si="16"/>
+        <f t="shared" si="29"/>
         <v>37</v>
       </c>
       <c r="H49" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>37</v>
       </c>
       <c r="I49" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100101</v>
       </c>
       <c r="J49" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>25</v>
       </c>
       <c r="L49" s="5" t="s">
@@ -3795,25 +4208,35 @@
         <v>1</v>
       </c>
       <c r="P49" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q49" s="3"/>
-      <c r="R49" s="3"/>
+        <v>190</v>
+      </c>
+      <c r="Q49" s="3">
+        <v>0</v>
+      </c>
+      <c r="R49" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S49" s="3"/>
       <c r="T49" s="3"/>
       <c r="U49" s="3"/>
       <c r="V49" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">37 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W49" s="3"/>
-      <c r="X49" s="3"/>
+      <c r="W49" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">37 =&gt; 0, </v>
+      </c>
+      <c r="X49" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">37 =&gt; op_nop, </v>
+      </c>
       <c r="Z49" s="16" t="str">
-        <f>"1 "&amp;H49&amp;" INSTRUCTION _"&amp;B49</f>
+        <f t="shared" si="27"/>
         <v>1 37 INSTRUCTION _LSL</v>
       </c>
       <c r="AA49" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B49&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," LSL"</v>
       </c>
     </row>
@@ -3830,20 +4253,20 @@
         <v>0</v>
       </c>
       <c r="F50" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="29"/>
         <v>38</v>
       </c>
       <c r="G50" s="14"/>
       <c r="H50" s="23">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>38</v>
       </c>
       <c r="I50" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100110</v>
       </c>
       <c r="J50" s="14" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>26</v>
       </c>
       <c r="K50" s="14"/>
@@ -3858,25 +4281,35 @@
       </c>
       <c r="O50" s="15"/>
       <c r="P50" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q50" s="3"/>
-      <c r="R50" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q50" s="3">
+        <v>0</v>
+      </c>
+      <c r="R50" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S50" s="14"/>
       <c r="T50" s="14"/>
       <c r="U50" s="14"/>
       <c r="V50" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">38 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W50" s="14"/>
-      <c r="X50" s="14"/>
+      <c r="W50" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">38 =&gt; 0, </v>
+      </c>
+      <c r="X50" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">38 =&gt; op_nop, </v>
+      </c>
       <c r="Z50" s="24" t="str">
-        <f>"1 "&amp;H50&amp;" INSTRUCTION _"&amp;B50</f>
+        <f t="shared" si="27"/>
         <v>1 38 INSTRUCTION _LSR</v>
       </c>
       <c r="AA50" s="24" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B50&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," LSR"</v>
       </c>
     </row>
@@ -3892,19 +4325,19 @@
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <f t="shared" si="16"/>
+        <f t="shared" si="29"/>
         <v>39</v>
       </c>
       <c r="H51" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>39</v>
       </c>
       <c r="I51" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0100111</v>
       </c>
       <c r="J51" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>27</v>
       </c>
       <c r="L51" s="5" t="s">
@@ -3917,25 +4350,35 @@
         <v>1</v>
       </c>
       <c r="P51" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q51" s="3"/>
-      <c r="R51" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q51" s="3">
+        <v>0</v>
+      </c>
+      <c r="R51" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S51" s="14"/>
       <c r="T51" s="14"/>
       <c r="U51" s="21"/>
       <c r="V51" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">39 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W51" s="21"/>
-      <c r="X51" s="21"/>
+      <c r="W51" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">39 =&gt; 0, </v>
+      </c>
+      <c r="X51" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">39 =&gt; op_nop, </v>
+      </c>
       <c r="Z51" s="16" t="str">
-        <f>"1 "&amp;H51&amp;" INSTRUCTION _"&amp;B51</f>
+        <f t="shared" si="27"/>
         <v>1 39 INSTRUCTION _XBYTE</v>
       </c>
       <c r="AA51" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B51&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," XBYTE"</v>
       </c>
     </row>
@@ -3951,19 +4394,19 @@
         <v>0</v>
       </c>
       <c r="F52" s="3">
-        <f t="shared" si="16"/>
+        <f t="shared" si="29"/>
         <v>40</v>
       </c>
       <c r="H52" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="23"/>
         <v>40</v>
       </c>
       <c r="I52" s="3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="24"/>
         <v>0101000</v>
       </c>
       <c r="J52" s="3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="25"/>
         <v>28</v>
       </c>
       <c r="L52" s="5" t="s">
@@ -3976,25 +4419,35 @@
         <v>1</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q52" s="3"/>
-      <c r="R52" s="14"/>
+        <v>190</v>
+      </c>
+      <c r="Q52" s="3">
+        <v>0</v>
+      </c>
+      <c r="R52" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S52" s="14"/>
       <c r="T52" s="14"/>
       <c r="U52" s="21"/>
       <c r="V52" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">40 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W52" s="21"/>
-      <c r="X52" s="21"/>
+      <c r="W52" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">40 =&gt; 0, </v>
+      </c>
+      <c r="X52" s="2" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">40 =&gt; op_nop, </v>
+      </c>
       <c r="Z52" s="16" t="str">
-        <f>"1 "&amp;H52&amp;" INSTRUCTION _"&amp;B52</f>
+        <f t="shared" si="27"/>
         <v>1 40 INSTRUCTION _XWORD</v>
       </c>
       <c r="AA52" s="16" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B52&amp;CHAR(34)</f>
+        <f t="shared" si="28"/>
         <v>," XWORD"</v>
       </c>
     </row>
@@ -4034,7 +4487,7 @@
         <v>41</v>
       </c>
       <c r="I55" s="3" t="str">
-        <f t="shared" ref="I55:I65" si="17">DEC2BIN(H55,7)</f>
+        <f t="shared" ref="I55:I65" si="30">DEC2BIN(H55,7)</f>
         <v>0101001</v>
       </c>
       <c r="J55" s="26" t="str">
@@ -4051,25 +4504,35 @@
       <c r="N55" s="26"/>
       <c r="O55" s="29"/>
       <c r="P55" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q55" s="26"/>
-      <c r="R55" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q55" s="26">
+        <v>4</v>
+      </c>
+      <c r="R55" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S55" s="26"/>
       <c r="T55" s="26"/>
       <c r="U55" s="26"/>
       <c r="V55" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">41 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W55" s="26"/>
-      <c r="X55" s="26"/>
+      <c r="W55" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">41 =&gt; 4, </v>
+      </c>
+      <c r="X55" s="2" t="str">
+        <f t="shared" ref="X55:X65" si="31">_xlfn.CONCAT($H55, " =&gt; ", R55, ", ")</f>
+        <v xml:space="preserve">41 =&gt; op_nop, </v>
+      </c>
       <c r="Z55" s="30" t="str">
-        <f>"1 "&amp;H55&amp;" INSTRUCTION _"&amp;B55</f>
+        <f t="shared" ref="Z55:Z65" si="32">"1 "&amp;H55&amp;" INSTRUCTION _"&amp;B55</f>
         <v>1 41 INSTRUCTION _MULTS</v>
       </c>
       <c r="AA55" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B55&amp;CHAR(34)</f>
+        <f t="shared" ref="AA55:AA65" si="33">CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B55&amp;CHAR(34)</f>
         <v>," MULTS"</v>
       </c>
     </row>
@@ -4094,7 +4557,7 @@
         <v>42</v>
       </c>
       <c r="I56" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101010</v>
       </c>
       <c r="J56" s="26" t="str">
@@ -4111,25 +4574,35 @@
       <c r="N56" s="26"/>
       <c r="O56" s="29"/>
       <c r="P56" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q56" s="26"/>
-      <c r="R56" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q56" s="26">
+        <v>4</v>
+      </c>
+      <c r="R56" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S56" s="26"/>
       <c r="T56" s="26"/>
       <c r="U56" s="26"/>
       <c r="V56" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">42 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W56" s="26"/>
-      <c r="X56" s="26"/>
+      <c r="W56" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">42 =&gt; 4, </v>
+      </c>
+      <c r="X56" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">42 =&gt; op_nop, </v>
+      </c>
       <c r="Z56" s="30" t="str">
-        <f>"1 "&amp;H56&amp;" INSTRUCTION _"&amp;B56</f>
+        <f t="shared" si="32"/>
         <v>1 42 INSTRUCTION _MULTU</v>
       </c>
       <c r="AA56" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B56&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," MULTU"</v>
       </c>
     </row>
@@ -4145,7 +4618,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="26">
-        <f t="shared" ref="F57:F64" si="18">F56+1</f>
+        <f t="shared" ref="F57:F64" si="34">F56+1</f>
         <v>43</v>
       </c>
       <c r="G57" s="26"/>
@@ -4154,7 +4627,7 @@
         <v>43</v>
       </c>
       <c r="I57" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101011</v>
       </c>
       <c r="J57" s="26" t="str">
@@ -4171,29 +4644,39 @@
       <c r="N57" s="26"/>
       <c r="O57" s="29"/>
       <c r="P57" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q57" s="26"/>
-      <c r="R57" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q57" s="26">
+        <v>200</v>
+      </c>
+      <c r="R57" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S57" s="26"/>
       <c r="T57" s="26"/>
       <c r="U57" s="26"/>
       <c r="V57" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">43 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W57" s="26"/>
-      <c r="X57" s="26"/>
+      <c r="W57" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">43 =&gt; 200, </v>
+      </c>
+      <c r="X57" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">43 =&gt; op_nop, </v>
+      </c>
       <c r="Z57" s="30" t="str">
-        <f>"1 "&amp;H57&amp;" INSTRUCTION _"&amp;B57</f>
+        <f t="shared" si="32"/>
         <v>1 43 INSTRUCTION _DIVS</v>
       </c>
       <c r="AA57" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B57&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," DIVS"</v>
       </c>
     </row>
-    <row r="58" spans="1:27" s="25" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:27" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B58" s="26" t="s">
         <v>129</v>
       </c>
@@ -4205,7 +4688,7 @@
         <v>0</v>
       </c>
       <c r="F58" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>44</v>
       </c>
       <c r="G58" s="26"/>
@@ -4214,7 +4697,7 @@
         <v>44</v>
       </c>
       <c r="I58" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101100</v>
       </c>
       <c r="J58" s="26" t="str">
@@ -4231,25 +4714,35 @@
       <c r="N58" s="26"/>
       <c r="O58" s="29"/>
       <c r="P58" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q58" s="26"/>
-      <c r="R58" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q58" s="26">
+        <v>200</v>
+      </c>
+      <c r="R58" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S58" s="26"/>
       <c r="T58" s="26"/>
       <c r="U58" s="26"/>
       <c r="V58" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">44 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W58" s="26"/>
-      <c r="X58" s="26"/>
+      <c r="W58" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">44 =&gt; 200, </v>
+      </c>
+      <c r="X58" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">44 =&gt; op_nop, </v>
+      </c>
       <c r="Z58" s="30" t="str">
-        <f>"1 "&amp;H58&amp;" INSTRUCTION _"&amp;B58</f>
+        <f t="shared" si="32"/>
         <v>1 44 INSTRUCTION _DIVU</v>
       </c>
       <c r="AA58" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B58&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," DIVU"</v>
       </c>
     </row>
@@ -4265,20 +4758,20 @@
         <v>0</v>
       </c>
       <c r="F59" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>45</v>
       </c>
       <c r="G59" s="26"/>
       <c r="H59" s="27">
-        <f t="shared" ref="H59:H64" si="19">F59+E59*64+D59*128</f>
+        <f t="shared" ref="H59:H64" si="35">F59+E59*64+D59*128</f>
         <v>45</v>
       </c>
       <c r="I59" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101101</v>
       </c>
       <c r="J59" s="26" t="str">
-        <f t="shared" ref="J59:J64" si="20">DEC2HEX(H59)</f>
+        <f t="shared" ref="J59:J64" si="36">DEC2HEX(H59)</f>
         <v>2D</v>
       </c>
       <c r="K59" s="26"/>
@@ -4291,25 +4784,35 @@
       <c r="N59" s="26"/>
       <c r="O59" s="29"/>
       <c r="P59" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q59" s="26"/>
-      <c r="R59" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q59" s="26">
+        <v>1</v>
+      </c>
+      <c r="R59" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S59" s="26"/>
       <c r="T59" s="26"/>
       <c r="U59" s="26"/>
       <c r="V59" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">45 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W59" s="26"/>
-      <c r="X59" s="26"/>
+      <c r="W59" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">45 =&gt; 1, </v>
+      </c>
+      <c r="X59" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">45 =&gt; op_nop, </v>
+      </c>
       <c r="Z59" s="30" t="str">
-        <f>"1 "&amp;H59&amp;" INSTRUCTION _"&amp;B59</f>
+        <f t="shared" si="32"/>
         <v>1 45 INSTRUCTION _FETCH.L</v>
       </c>
       <c r="AA59" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B59&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," FETCH.L"</v>
       </c>
     </row>
@@ -4325,20 +4828,20 @@
         <v>0</v>
       </c>
       <c r="F60" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>46</v>
       </c>
       <c r="G60" s="26"/>
       <c r="H60" s="27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="35"/>
         <v>46</v>
       </c>
       <c r="I60" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101110</v>
       </c>
       <c r="J60" s="26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="36"/>
         <v>2E</v>
       </c>
       <c r="K60" s="26"/>
@@ -4351,25 +4854,35 @@
       <c r="N60" s="26"/>
       <c r="O60" s="29"/>
       <c r="P60" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q60" s="26"/>
-      <c r="R60" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q60" s="26">
+        <v>1</v>
+      </c>
+      <c r="R60" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S60" s="26"/>
       <c r="T60" s="26"/>
       <c r="U60" s="26"/>
       <c r="V60" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">46 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W60" s="26"/>
-      <c r="X60" s="26"/>
+      <c r="W60" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">46 =&gt; 1, </v>
+      </c>
+      <c r="X60" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">46 =&gt; op_nop, </v>
+      </c>
       <c r="Z60" s="30" t="str">
-        <f>"1 "&amp;H60&amp;" INSTRUCTION _"&amp;B60</f>
+        <f t="shared" si="32"/>
         <v>1 46 INSTRUCTION _STORE.L</v>
       </c>
       <c r="AA60" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B60&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," STORE.L"</v>
       </c>
     </row>
@@ -4385,20 +4898,20 @@
         <v>0</v>
       </c>
       <c r="F61" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>47</v>
       </c>
       <c r="G61" s="26"/>
       <c r="H61" s="27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="35"/>
         <v>47</v>
       </c>
       <c r="I61" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0101111</v>
       </c>
       <c r="J61" s="26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="36"/>
         <v>2F</v>
       </c>
       <c r="K61" s="26"/>
@@ -4411,25 +4924,35 @@
       <c r="N61" s="26"/>
       <c r="O61" s="29"/>
       <c r="P61" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q61" s="26"/>
-      <c r="R61" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q61" s="26">
+        <v>1</v>
+      </c>
+      <c r="R61" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S61" s="26"/>
       <c r="T61" s="26"/>
       <c r="U61" s="26"/>
       <c r="V61" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">47 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W61" s="26"/>
-      <c r="X61" s="26"/>
+      <c r="W61" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">47 =&gt; 1, </v>
+      </c>
+      <c r="X61" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">47 =&gt; op_nop, </v>
+      </c>
       <c r="Z61" s="30" t="str">
-        <f>"1 "&amp;H61&amp;" INSTRUCTION _"&amp;B61</f>
+        <f t="shared" si="32"/>
         <v>1 47 INSTRUCTION _FETCH.W</v>
       </c>
       <c r="AA61" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B61&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," FETCH.W"</v>
       </c>
     </row>
@@ -4445,20 +4968,20 @@
         <v>0</v>
       </c>
       <c r="F62" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>48</v>
       </c>
       <c r="G62" s="26"/>
       <c r="H62" s="27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="35"/>
         <v>48</v>
       </c>
       <c r="I62" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0110000</v>
       </c>
       <c r="J62" s="26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="36"/>
         <v>30</v>
       </c>
       <c r="K62" s="26"/>
@@ -4471,25 +4994,35 @@
       <c r="N62" s="26"/>
       <c r="O62" s="29"/>
       <c r="P62" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q62" s="26"/>
-      <c r="R62" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q62" s="26">
+        <v>1</v>
+      </c>
+      <c r="R62" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S62" s="26"/>
       <c r="T62" s="26"/>
       <c r="U62" s="26"/>
       <c r="V62" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">48 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W62" s="26"/>
-      <c r="X62" s="26"/>
+      <c r="W62" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">48 =&gt; 1, </v>
+      </c>
+      <c r="X62" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">48 =&gt; op_nop, </v>
+      </c>
       <c r="Z62" s="30" t="str">
-        <f>"1 "&amp;H62&amp;" INSTRUCTION _"&amp;B62</f>
+        <f t="shared" si="32"/>
         <v>1 48 INSTRUCTION _STORE.W</v>
       </c>
       <c r="AA62" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B62&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," STORE.W"</v>
       </c>
     </row>
@@ -4505,20 +5038,20 @@
         <v>0</v>
       </c>
       <c r="F63" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>49</v>
       </c>
       <c r="G63" s="26"/>
       <c r="H63" s="27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="35"/>
         <v>49</v>
       </c>
       <c r="I63" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0110001</v>
       </c>
       <c r="J63" s="26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="36"/>
         <v>31</v>
       </c>
       <c r="K63" s="26"/>
@@ -4531,25 +5064,35 @@
       <c r="N63" s="26"/>
       <c r="O63" s="29"/>
       <c r="P63" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q63" s="26"/>
-      <c r="R63" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q63" s="26">
+        <v>1</v>
+      </c>
+      <c r="R63" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S63" s="26"/>
       <c r="T63" s="26"/>
       <c r="U63" s="26"/>
       <c r="V63" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">49 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W63" s="26"/>
-      <c r="X63" s="26"/>
+      <c r="W63" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">49 =&gt; 1, </v>
+      </c>
+      <c r="X63" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">49 =&gt; op_nop, </v>
+      </c>
       <c r="Z63" s="30" t="str">
-        <f>"1 "&amp;H63&amp;" INSTRUCTION _"&amp;B63</f>
+        <f t="shared" si="32"/>
         <v>1 49 INSTRUCTION _FETCH.B</v>
       </c>
       <c r="AA63" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B63&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," FETCH.B"</v>
       </c>
     </row>
@@ -4565,20 +5108,20 @@
         <v>0</v>
       </c>
       <c r="F64" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="34"/>
         <v>50</v>
       </c>
       <c r="G64" s="26"/>
       <c r="H64" s="27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="35"/>
         <v>50</v>
       </c>
       <c r="I64" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0110010</v>
       </c>
       <c r="J64" s="26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="36"/>
         <v>32</v>
       </c>
       <c r="K64" s="26"/>
@@ -4591,31 +5134,41 @@
       <c r="N64" s="26"/>
       <c r="O64" s="29"/>
       <c r="P64" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q64" s="26"/>
-      <c r="R64" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q64" s="26">
+        <v>1</v>
+      </c>
+      <c r="R64" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S64" s="26"/>
       <c r="T64" s="26"/>
       <c r="U64" s="26"/>
       <c r="V64" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">50 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W64" s="26"/>
-      <c r="X64" s="26"/>
+      <c r="W64" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">50 =&gt; 1, </v>
+      </c>
+      <c r="X64" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">50 =&gt; op_nop, </v>
+      </c>
       <c r="Z64" s="30" t="str">
-        <f>"1 "&amp;H64&amp;" INSTRUCTION _"&amp;B64</f>
+        <f t="shared" si="32"/>
         <v>1 50 INSTRUCTION _STORE.B</v>
       </c>
       <c r="AA64" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B64&amp;CHAR(34)</f>
+        <f t="shared" si="33"/>
         <v>," STORE.B"</v>
       </c>
     </row>
     <row r="65" spans="1:27" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B65" s="26" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="C65" s="26"/>
       <c r="D65" s="26">
@@ -4634,7 +5187,7 @@
         <v>51</v>
       </c>
       <c r="I65" s="3" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="30"/>
         <v>0110011</v>
       </c>
       <c r="J65" s="26" t="str">
@@ -4643,36 +5196,46 @@
       </c>
       <c r="K65" s="26"/>
       <c r="L65" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="M65" s="25" t="s">
         <v>151</v>
-      </c>
-      <c r="M65" s="25" t="s">
-        <v>152</v>
       </c>
       <c r="N65" s="26">
         <v>2</v>
       </c>
       <c r="O65" s="29"/>
       <c r="P65" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q65" s="26"/>
-      <c r="R65" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="Q65" s="26">
+        <v>0</v>
+      </c>
+      <c r="R65" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S65" s="26"/>
       <c r="T65" s="26"/>
       <c r="U65" s="26"/>
       <c r="V65" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">51 =&gt; pf_nxt_1, </v>
       </c>
-      <c r="W65" s="26"/>
-      <c r="X65" s="26"/>
+      <c r="W65" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">51 =&gt; 0, </v>
+      </c>
+      <c r="X65" s="2" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">51 =&gt; op_nop, </v>
+      </c>
       <c r="Z65" s="30" t="str">
-        <f>"1 "&amp;H65&amp;" INSTRUCTION _"&amp;B65</f>
-        <v>1 51 INSTRUCTION _?DUP</v>
+        <f t="shared" si="32"/>
+        <v>1 51 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA65" s="30" t="str">
-        <f>CHAR(44)&amp;CHAR(34)&amp;CHAR(32)&amp;B65&amp;CHAR(34)</f>
-        <v>," ?DUP"</v>
+        <f t="shared" si="33"/>
+        <v>," UNUSED"</v>
       </c>
     </row>
     <row r="66" spans="1:27" s="32" customFormat="1" x14ac:dyDescent="0.2">
@@ -4693,12 +5256,13 @@
       <c r="Q66" s="36"/>
       <c r="R66" s="33"/>
       <c r="V66" s="2"/>
+      <c r="W66" s="2"/>
       <c r="Z66" s="16"/>
       <c r="AA66" s="37"/>
     </row>
     <row r="67" spans="1:27" s="32" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B67" s="33"/>
       <c r="C67" s="33"/>
@@ -4717,12 +5281,13 @@
       <c r="Q67" s="36"/>
       <c r="R67" s="33"/>
       <c r="V67" s="2"/>
+      <c r="W67" s="2"/>
       <c r="Z67" s="16"/>
       <c r="AA67" s="37"/>
     </row>
     <row r="68" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B68" s="40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C68" s="40"/>
       <c r="D68" s="40">
@@ -4737,42 +5302,52 @@
       </c>
       <c r="G68" s="40"/>
       <c r="H68" s="42">
-        <f t="shared" ref="H68:H77" si="21">F68+E68*64+D68*128</f>
+        <f t="shared" ref="H68:H77" si="37">F68+E68*64+D68*128</f>
         <v>52</v>
       </c>
       <c r="I68" s="3" t="str">
-        <f t="shared" ref="I68:I77" si="22">DEC2BIN(H68,7)</f>
+        <f t="shared" ref="I68:I77" si="38">DEC2BIN(H68,7)</f>
         <v>0110100</v>
       </c>
       <c r="J68" s="40" t="str">
-        <f t="shared" ref="J68:J77" si="23">DEC2HEX(H68)</f>
+        <f t="shared" ref="J68:J77" si="39">DEC2HEX(H68)</f>
         <v>34</v>
       </c>
       <c r="K68" s="40"/>
       <c r="L68" s="43" t="s">
+        <v>154</v>
+      </c>
+      <c r="M68" s="39" t="s">
         <v>155</v>
-      </c>
-      <c r="M68" s="39" t="s">
-        <v>156</v>
       </c>
       <c r="N68" s="40"/>
       <c r="O68" s="38"/>
       <c r="P68" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q68" s="40"/>
-      <c r="R68" s="40"/>
+        <v>191</v>
+      </c>
+      <c r="Q68" s="40">
+        <v>0</v>
+      </c>
+      <c r="R68" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S68" s="40"/>
       <c r="T68" s="40"/>
       <c r="U68" s="40"/>
       <c r="V68" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">52 =&gt; pf_nxt_2, </v>
       </c>
-      <c r="W68" s="40"/>
-      <c r="X68" s="40"/>
+      <c r="W68" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">52 =&gt; 0, </v>
+      </c>
+      <c r="X68" s="2" t="str">
+        <f t="shared" ref="X68:X77" si="40">_xlfn.CONCAT($H68, " =&gt; ", R68, ", ")</f>
+        <v xml:space="preserve">52 =&gt; op_nop, </v>
+      </c>
       <c r="Z68" s="44" t="str">
-        <f>"1 "&amp;H68&amp;" INSTRUCTION _"&amp;B68</f>
+        <f t="shared" ref="Z68:Z77" si="41">"1 "&amp;H68&amp;" INSTRUCTION _"&amp;B68</f>
         <v>1 52 INSTRUCTION _#.B</v>
       </c>
       <c r="AA68" s="44" t="str">
@@ -4782,7 +5357,7 @@
     </row>
     <row r="69" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B69" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C69" s="40"/>
       <c r="D69" s="40">
@@ -4792,47 +5367,57 @@
         <v>0</v>
       </c>
       <c r="F69" s="40">
-        <f t="shared" ref="F69:F77" si="24">F68+1</f>
+        <f t="shared" ref="F69:F77" si="42">F68+1</f>
         <v>53</v>
       </c>
       <c r="G69" s="40"/>
       <c r="H69" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>53</v>
       </c>
       <c r="I69" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0110101</v>
       </c>
       <c r="J69" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>35</v>
       </c>
       <c r="K69" s="40"/>
       <c r="L69" s="43" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M69" s="39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="N69" s="40"/>
       <c r="O69" s="38"/>
       <c r="P69" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q69" s="40"/>
-      <c r="R69" s="40"/>
+        <v>192</v>
+      </c>
+      <c r="Q69" s="40">
+        <v>0</v>
+      </c>
+      <c r="R69" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S69" s="40"/>
       <c r="T69" s="40"/>
       <c r="U69" s="40"/>
       <c r="V69" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">53 =&gt; pf_nxt_3, </v>
       </c>
-      <c r="W69" s="40"/>
-      <c r="X69" s="40"/>
+      <c r="W69" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">53 =&gt; 0, </v>
+      </c>
+      <c r="X69" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">53 =&gt; op_nop, </v>
+      </c>
       <c r="Z69" s="44" t="str">
-        <f>"1 "&amp;H69&amp;" INSTRUCTION _"&amp;B69</f>
+        <f t="shared" si="41"/>
         <v>1 53 INSTRUCTION _#.W</v>
       </c>
       <c r="AA69" s="44" t="str">
@@ -4842,7 +5427,7 @@
     </row>
     <row r="70" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B70" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C70" s="40"/>
       <c r="D70" s="40">
@@ -4852,47 +5437,57 @@
         <v>0</v>
       </c>
       <c r="F70" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>54</v>
       </c>
       <c r="G70" s="40"/>
       <c r="H70" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>54</v>
       </c>
       <c r="I70" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0110110</v>
       </c>
       <c r="J70" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>36</v>
       </c>
       <c r="K70" s="40"/>
       <c r="L70" s="43" t="s">
+        <v>159</v>
+      </c>
+      <c r="M70" s="39" t="s">
         <v>160</v>
-      </c>
-      <c r="M70" s="39" t="s">
-        <v>161</v>
       </c>
       <c r="N70" s="40"/>
       <c r="O70" s="38"/>
       <c r="P70" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="Q70" s="40"/>
-      <c r="R70" s="40"/>
+        <v>193</v>
+      </c>
+      <c r="Q70" s="40">
+        <v>0</v>
+      </c>
+      <c r="R70" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S70" s="40"/>
       <c r="T70" s="40"/>
       <c r="U70" s="40"/>
       <c r="V70" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v xml:space="preserve">54 =&gt; pf_nxt_5, </v>
       </c>
-      <c r="W70" s="40"/>
-      <c r="X70" s="40"/>
+      <c r="W70" s="2" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve">54 =&gt; 0, </v>
+      </c>
+      <c r="X70" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">54 =&gt; op_nop, </v>
+      </c>
       <c r="Z70" s="44" t="str">
-        <f>"1 "&amp;H70&amp;" INSTRUCTION _"&amp;B70</f>
+        <f t="shared" si="41"/>
         <v>1 54 INSTRUCTION _#.L</v>
       </c>
       <c r="AA70" s="44" t="str">
@@ -4902,7 +5497,7 @@
     </row>
     <row r="71" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B71" s="40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C71" s="40"/>
       <c r="D71" s="40">
@@ -4912,47 +5507,57 @@
         <v>0</v>
       </c>
       <c r="F71" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>55</v>
       </c>
       <c r="G71" s="40"/>
       <c r="H71" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>55</v>
       </c>
       <c r="I71" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0110111</v>
       </c>
       <c r="J71" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>37</v>
       </c>
       <c r="K71" s="40"/>
       <c r="L71" s="43" t="s">
+        <v>162</v>
+      </c>
+      <c r="M71" s="39" t="s">
         <v>163</v>
-      </c>
-      <c r="M71" s="39" t="s">
-        <v>164</v>
       </c>
       <c r="N71" s="40"/>
       <c r="O71" s="38"/>
       <c r="P71" s="40" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q71" s="40"/>
-      <c r="R71" s="40"/>
+        <v>194</v>
+      </c>
+      <c r="Q71" s="40">
+        <v>0</v>
+      </c>
+      <c r="R71" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S71" s="40"/>
       <c r="T71" s="40"/>
       <c r="U71" s="40"/>
       <c r="V71" s="2" t="str">
-        <f t="shared" ref="V71:V91" si="25">_xlfn.CONCAT(H71, " =&gt; ", P71, ", ")</f>
+        <f t="shared" ref="V71:V81" si="43">_xlfn.CONCAT(H71, " =&gt; ", P71, ", ")</f>
         <v xml:space="preserve">55 =&gt; pf_jmp, </v>
       </c>
-      <c r="W71" s="40"/>
-      <c r="X71" s="40"/>
+      <c r="W71" s="2" t="str">
+        <f t="shared" ref="W71:W81" si="44">_xlfn.CONCAT(H71, " =&gt; ", Q71, ", ")</f>
+        <v xml:space="preserve">55 =&gt; 0, </v>
+      </c>
+      <c r="X71" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">55 =&gt; op_nop, </v>
+      </c>
       <c r="Z71" s="44" t="str">
-        <f>"1 "&amp;H71&amp;" INSTRUCTION _"&amp;B71</f>
+        <f t="shared" si="41"/>
         <v>1 55 INSTRUCTION _JMP</v>
       </c>
       <c r="AA71" s="44" t="str">
@@ -4962,7 +5567,7 @@
     </row>
     <row r="72" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B72" s="40" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C72" s="40"/>
       <c r="D72" s="40">
@@ -4972,56 +5577,66 @@
         <v>0</v>
       </c>
       <c r="F72" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>56</v>
       </c>
       <c r="G72" s="40"/>
       <c r="H72" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>56</v>
       </c>
       <c r="I72" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111000</v>
       </c>
       <c r="J72" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>38</v>
       </c>
       <c r="K72" s="40"/>
       <c r="L72" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="M72" s="39" t="s">
         <v>166</v>
-      </c>
-      <c r="M72" s="39" t="s">
-        <v>167</v>
       </c>
       <c r="N72" s="40"/>
       <c r="O72" s="38"/>
       <c r="P72" s="40" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q72" s="40"/>
-      <c r="R72" s="40"/>
+        <v>195</v>
+      </c>
+      <c r="Q72" s="40">
+        <v>0</v>
+      </c>
+      <c r="R72" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="S72" s="40"/>
       <c r="T72" s="40"/>
       <c r="U72" s="40"/>
       <c r="V72" s="2" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="43"/>
         <v xml:space="preserve">56 =&gt; pf_jsl, </v>
       </c>
-      <c r="W72" s="40"/>
-      <c r="X72" s="40"/>
+      <c r="W72" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">56 =&gt; 0, </v>
+      </c>
+      <c r="X72" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">56 =&gt; op_psh, </v>
+      </c>
       <c r="Z72" s="44" t="str">
-        <f>"1 "&amp;H72&amp;" INSTRUCTION _"&amp;B72</f>
+        <f t="shared" si="41"/>
         <v>1 56 INSTRUCTION _JSL</v>
       </c>
       <c r="AA72" s="44" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="73" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B73" s="40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C73" s="40"/>
       <c r="D73" s="40">
@@ -5031,47 +5646,57 @@
         <v>0</v>
       </c>
       <c r="F73" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>57</v>
       </c>
       <c r="G73" s="40"/>
       <c r="H73" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>57</v>
       </c>
       <c r="I73" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111001</v>
       </c>
       <c r="J73" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>39</v>
       </c>
       <c r="K73" s="40"/>
       <c r="L73" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="M73" s="39" t="s">
         <v>170</v>
-      </c>
-      <c r="M73" s="39" t="s">
-        <v>171</v>
       </c>
       <c r="N73" s="40"/>
       <c r="O73" s="38"/>
       <c r="P73" s="40" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q73" s="40"/>
-      <c r="R73" s="40"/>
+        <v>196</v>
+      </c>
+      <c r="Q73" s="40">
+        <v>0</v>
+      </c>
+      <c r="R73" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="S73" s="40"/>
       <c r="T73" s="40"/>
       <c r="U73" s="40"/>
       <c r="V73" s="2" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="43"/>
         <v xml:space="preserve">57 =&gt; pf_jsr, </v>
       </c>
-      <c r="W73" s="40"/>
-      <c r="X73" s="40"/>
+      <c r="W73" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">57 =&gt; 0, </v>
+      </c>
+      <c r="X73" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">57 =&gt; op_psh, </v>
+      </c>
       <c r="Z73" s="44" t="str">
-        <f>"1 "&amp;H73&amp;" INSTRUCTION _"&amp;B73</f>
+        <f t="shared" si="41"/>
         <v>1 57 INSTRUCTION _JSR</v>
       </c>
       <c r="AA73" s="44" t="str">
@@ -5081,7 +5706,7 @@
     </row>
     <row r="74" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B74" s="40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C74" s="40"/>
       <c r="D74" s="40">
@@ -5091,20 +5716,20 @@
         <v>0</v>
       </c>
       <c r="F74" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>58</v>
       </c>
       <c r="G74" s="40"/>
       <c r="H74" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>58</v>
       </c>
       <c r="I74" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111010</v>
       </c>
       <c r="J74" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>3A</v>
       </c>
       <c r="K74" s="40"/>
@@ -5112,24 +5737,36 @@
         <v>16</v>
       </c>
       <c r="M74" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N74" s="40"/>
       <c r="O74" s="38"/>
-      <c r="P74" s="40"/>
-      <c r="Q74" s="40"/>
-      <c r="R74" s="40"/>
+      <c r="P74" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q74" s="3">
+        <v>0</v>
+      </c>
+      <c r="R74" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S74" s="40"/>
       <c r="T74" s="40"/>
       <c r="U74" s="40"/>
       <c r="V74" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">58 =&gt; , </v>
-      </c>
-      <c r="W74" s="40"/>
-      <c r="X74" s="40"/>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">58 =&gt; pf_nxt_1, </v>
+      </c>
+      <c r="W74" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">58 =&gt; 0, </v>
+      </c>
+      <c r="X74" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">58 =&gt; op_nop, </v>
+      </c>
       <c r="Z74" s="44" t="str">
-        <f>"1 "&amp;H74&amp;" INSTRUCTION _"&amp;B74</f>
+        <f t="shared" si="41"/>
         <v>1 58 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA74" s="44" t="str">
@@ -5139,7 +5776,7 @@
     </row>
     <row r="75" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B75" s="40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C75" s="40"/>
       <c r="D75" s="40">
@@ -5149,20 +5786,20 @@
         <v>0</v>
       </c>
       <c r="F75" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>59</v>
       </c>
       <c r="G75" s="40"/>
       <c r="H75" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>59</v>
       </c>
       <c r="I75" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111011</v>
       </c>
       <c r="J75" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>3B</v>
       </c>
       <c r="K75" s="40"/>
@@ -5170,24 +5807,36 @@
         <v>16</v>
       </c>
       <c r="M75" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N75" s="40"/>
       <c r="O75" s="38"/>
-      <c r="P75" s="40"/>
-      <c r="Q75" s="40"/>
-      <c r="R75" s="40"/>
+      <c r="P75" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q75" s="3">
+        <v>0</v>
+      </c>
+      <c r="R75" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S75" s="40"/>
       <c r="T75" s="40"/>
       <c r="U75" s="40"/>
       <c r="V75" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">59 =&gt; , </v>
-      </c>
-      <c r="W75" s="40"/>
-      <c r="X75" s="40"/>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">59 =&gt; pf_nxt_1, </v>
+      </c>
+      <c r="W75" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">59 =&gt; 0, </v>
+      </c>
+      <c r="X75" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">59 =&gt; op_nop, </v>
+      </c>
       <c r="Z75" s="44" t="str">
-        <f>"1 "&amp;H75&amp;" INSTRUCTION _"&amp;B75</f>
+        <f t="shared" si="41"/>
         <v>1 59 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA75" s="44" t="str">
@@ -5197,7 +5846,7 @@
     </row>
     <row r="76" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B76" s="40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C76" s="40"/>
       <c r="D76" s="40">
@@ -5207,20 +5856,20 @@
         <v>0</v>
       </c>
       <c r="F76" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>60</v>
       </c>
       <c r="G76" s="40"/>
       <c r="H76" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>60</v>
       </c>
       <c r="I76" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111100</v>
       </c>
       <c r="J76" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>3C</v>
       </c>
       <c r="K76" s="40"/>
@@ -5228,24 +5877,36 @@
         <v>16</v>
       </c>
       <c r="M76" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N76" s="40"/>
       <c r="O76" s="38"/>
-      <c r="P76" s="40"/>
-      <c r="Q76" s="40"/>
-      <c r="R76" s="40"/>
+      <c r="P76" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q76" s="3">
+        <v>0</v>
+      </c>
+      <c r="R76" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S76" s="40"/>
       <c r="T76" s="40"/>
       <c r="U76" s="40"/>
       <c r="V76" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">60 =&gt; , </v>
-      </c>
-      <c r="W76" s="40"/>
-      <c r="X76" s="40"/>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">60 =&gt; pf_nxt_1, </v>
+      </c>
+      <c r="W76" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">60 =&gt; 0, </v>
+      </c>
+      <c r="X76" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">60 =&gt; op_nop, </v>
+      </c>
       <c r="Z76" s="44" t="str">
-        <f>"1 "&amp;H76&amp;" INSTRUCTION _"&amp;B76</f>
+        <f t="shared" si="41"/>
         <v>1 60 INSTRUCTION _UNUSED</v>
       </c>
       <c r="AA76" s="44" t="str">
@@ -5255,7 +5916,7 @@
     </row>
     <row r="77" spans="1:27" s="39" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B77" s="40" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C77" s="40"/>
       <c r="D77" s="40">
@@ -5265,20 +5926,20 @@
         <v>0</v>
       </c>
       <c r="F77" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="42"/>
         <v>61</v>
       </c>
       <c r="G77" s="40"/>
       <c r="H77" s="42">
-        <f t="shared" si="21"/>
+        <f t="shared" si="37"/>
         <v>61</v>
       </c>
       <c r="I77" s="3" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="38"/>
         <v>0111101</v>
       </c>
       <c r="J77" s="40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="39"/>
         <v>3D</v>
       </c>
       <c r="K77" s="40"/>
@@ -5286,26 +5947,36 @@
         <v>16</v>
       </c>
       <c r="M77" s="39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="N77" s="40"/>
       <c r="O77" s="38"/>
       <c r="P77" s="40" t="s">
-        <v>200</v>
-      </c>
-      <c r="Q77" s="40"/>
-      <c r="R77" s="40"/>
+        <v>197</v>
+      </c>
+      <c r="Q77" s="40">
+        <v>0</v>
+      </c>
+      <c r="R77" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S77" s="40"/>
       <c r="T77" s="40"/>
       <c r="U77" s="40"/>
       <c r="V77" s="2" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="43"/>
         <v xml:space="preserve">61 =&gt; ps_slp, </v>
       </c>
-      <c r="W77" s="40"/>
-      <c r="X77" s="40"/>
+      <c r="W77" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">61 =&gt; 0, </v>
+      </c>
+      <c r="X77" s="2" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">61 =&gt; op_nop, </v>
+      </c>
       <c r="Z77" s="44" t="str">
-        <f>"1 "&amp;H77&amp;" INSTRUCTION _"&amp;B77</f>
+        <f t="shared" si="41"/>
         <v>1 61 INSTRUCTION _PAUSE</v>
       </c>
       <c r="AA77" s="44" t="str">
@@ -5334,14 +6005,14 @@
       <c r="T78" s="40"/>
       <c r="U78" s="40"/>
       <c r="V78" s="2"/>
-      <c r="W78" s="40"/>
+      <c r="W78" s="2"/>
       <c r="X78" s="40"/>
       <c r="Z78" s="44"/>
       <c r="AA78" s="44"/>
     </row>
     <row r="79" spans="1:27" s="17" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B79" s="14"/>
       <c r="C79" s="14"/>
@@ -5363,14 +6034,14 @@
       <c r="T79" s="14"/>
       <c r="U79" s="14"/>
       <c r="V79" s="2"/>
-      <c r="W79" s="14"/>
+      <c r="W79" s="2"/>
       <c r="X79" s="14"/>
       <c r="Z79" s="24"/>
       <c r="AA79" s="24"/>
     </row>
     <row r="80" spans="1:27" s="17" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B80" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C80" s="14"/>
       <c r="D80" s="14">
@@ -5388,7 +6059,7 @@
         <v>62</v>
       </c>
       <c r="I80" s="14" t="str">
-        <f t="shared" ref="I80:I81" si="26">DEC2BIN(H80,7)</f>
+        <f t="shared" ref="I80:I81" si="45">DEC2BIN(H80,7)</f>
         <v>0111110</v>
       </c>
       <c r="J80" s="14" t="str">
@@ -5399,18 +6070,30 @@
       <c r="L80" s="19"/>
       <c r="N80" s="14"/>
       <c r="O80" s="15"/>
-      <c r="P80" s="3"/>
-      <c r="Q80" s="3"/>
-      <c r="R80" s="14"/>
+      <c r="P80" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q80" s="3">
+        <v>0</v>
+      </c>
+      <c r="R80" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S80" s="14"/>
       <c r="T80" s="14"/>
       <c r="U80" s="2"/>
       <c r="V80" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">62 =&gt; , </v>
-      </c>
-      <c r="W80" s="2"/>
-      <c r="X80" s="2"/>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">62 =&gt; pf_nxt_1, </v>
+      </c>
+      <c r="W80" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">62 =&gt; 0, </v>
+      </c>
+      <c r="X80" s="2" t="str">
+        <f t="shared" ref="X80:X81" si="46">_xlfn.CONCAT($H80, " =&gt; ", R80, ", ")</f>
+        <v xml:space="preserve">62 =&gt; op_nop, </v>
+      </c>
       <c r="Z80" s="44" t="str">
         <f>"1 "&amp;H80&amp;" INSTRUCTION _"&amp;B80</f>
         <v>1 62 INSTRUCTION _UNUSED</v>
@@ -5422,7 +6105,7 @@
     </row>
     <row r="81" spans="1:27" s="17" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B81" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C81" s="14"/>
       <c r="D81" s="14">
@@ -5436,33 +6119,45 @@
       </c>
       <c r="G81" s="14"/>
       <c r="H81" s="23">
-        <f t="shared" ref="H81" si="27">F81+E81*64+D81*128</f>
+        <f t="shared" ref="H81" si="47">F81+E81*64+D81*128</f>
         <v>63</v>
       </c>
       <c r="I81" s="14" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="45"/>
         <v>0111111</v>
       </c>
       <c r="J81" s="14" t="str">
-        <f t="shared" ref="J81" si="28">DEC2HEX(H81)</f>
+        <f t="shared" ref="J81" si="48">DEC2HEX(H81)</f>
         <v>3F</v>
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="19"/>
       <c r="N81" s="14"/>
       <c r="O81" s="15"/>
-      <c r="P81" s="3"/>
-      <c r="Q81" s="3"/>
-      <c r="R81" s="14"/>
+      <c r="P81" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q81" s="3">
+        <v>0</v>
+      </c>
+      <c r="R81" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S81" s="14"/>
       <c r="T81" s="14"/>
       <c r="U81" s="2"/>
       <c r="V81" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">63 =&gt; , </v>
-      </c>
-      <c r="W81" s="2"/>
-      <c r="X81" s="2"/>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">63 =&gt; pf_nxt_1, </v>
+      </c>
+      <c r="W81" s="2" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">63 =&gt; 0, </v>
+      </c>
+      <c r="X81" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">63 =&gt; op_nop, </v>
+      </c>
       <c r="Z81" s="44" t="str">
         <f>"1 "&amp;H81&amp;" INSTRUCTION _"&amp;B81</f>
         <v>1 63 INSTRUCTION _UNUSED</v>
@@ -5493,7 +6188,7 @@
     </row>
     <row r="83" spans="1:27" s="51" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="49" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B83" s="46"/>
       <c r="C83" s="46"/>
@@ -5530,11 +6225,11 @@
       </c>
       <c r="G84" s="46"/>
       <c r="H84" s="47">
-        <f t="shared" ref="H84" si="29">F84+E84*64+D84*128</f>
+        <f t="shared" ref="H84" si="49">F84+E84*64+D84*128</f>
         <v>64</v>
       </c>
       <c r="I84" s="46" t="str">
-        <f t="shared" ref="I84:I86" si="30">DEC2BIN(H84,7)</f>
+        <f t="shared" ref="I84:I86" si="50">DEC2BIN(H84,7)</f>
         <v>1000000</v>
       </c>
       <c r="J84" s="46" t="str">
@@ -5555,15 +6250,12 @@
       <c r="R84" s="46"/>
       <c r="S84" s="46"/>
       <c r="T84" s="46"/>
-      <c r="V84" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">64 =&gt; , </v>
-      </c>
+      <c r="V84" s="2"/>
       <c r="Z84" s="52"/>
     </row>
     <row r="85" spans="1:27" s="51" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B85" s="46" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C85" s="46"/>
       <c r="D85" s="46">
@@ -5581,7 +6273,7 @@
         <v>65</v>
       </c>
       <c r="I85" s="46" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="50"/>
         <v>1000001</v>
       </c>
       <c r="J85" s="46" t="str">
@@ -5590,10 +6282,10 @@
       </c>
       <c r="K85" s="46"/>
       <c r="L85" s="50" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M85" s="51" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N85" s="46"/>
       <c r="O85" s="49"/>
@@ -5603,10 +6295,7 @@
       <c r="S85" s="46"/>
       <c r="T85" s="46"/>
       <c r="U85" s="46"/>
-      <c r="V85" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">65 =&gt; , </v>
-      </c>
+      <c r="V85" s="2"/>
       <c r="W85" s="46"/>
       <c r="X85" s="46"/>
       <c r="Z85" s="53"/>
@@ -5614,7 +6303,7 @@
     </row>
     <row r="86" spans="1:27" s="51" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B86" s="46" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C86" s="46"/>
       <c r="D86" s="46">
@@ -5632,7 +6321,7 @@
         <v>66</v>
       </c>
       <c r="I86" s="46" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="50"/>
         <v>1000010</v>
       </c>
       <c r="J86" s="46" t="str">
@@ -5644,7 +6333,7 @@
         <v>64</v>
       </c>
       <c r="M86" s="51" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="N86" s="46"/>
       <c r="O86" s="49"/>
@@ -5654,10 +6343,7 @@
       <c r="S86" s="46"/>
       <c r="T86" s="46"/>
       <c r="U86" s="46"/>
-      <c r="V86" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">66 =&gt; , </v>
-      </c>
+      <c r="V86" s="2"/>
       <c r="W86" s="46"/>
       <c r="X86" s="46"/>
       <c r="Z86" s="53"/>
@@ -5668,7 +6354,7 @@
     </row>
     <row r="88" spans="1:27" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="54" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B88" s="55"/>
       <c r="C88" s="55"/>
@@ -5690,7 +6376,7 @@
     </row>
     <row r="89" spans="1:27" s="54" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B89" s="55" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C89" s="55"/>
       <c r="D89" s="55">
@@ -5704,33 +6390,36 @@
       </c>
       <c r="G89" s="55"/>
       <c r="H89" s="56">
-        <f t="shared" ref="H89:H91" si="31">F89+E89*64+D89*128</f>
+        <f t="shared" ref="H89:H91" si="51">F89+E89*64+D89*128</f>
         <v>64</v>
       </c>
       <c r="I89" s="55"/>
       <c r="J89" s="55" t="str">
-        <f t="shared" ref="J89:J91" si="32">DEC2HEX(H89)</f>
+        <f t="shared" ref="J89:J91" si="52">DEC2HEX(H89)</f>
         <v>40</v>
       </c>
       <c r="K89" s="55"/>
       <c r="L89" s="60" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M89" s="54" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="N89" s="55"/>
       <c r="O89" s="58"/>
-      <c r="P89" s="58"/>
-      <c r="Q89" s="58"/>
-      <c r="R89" s="55"/>
+      <c r="P89" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q89" s="3">
+        <v>0</v>
+      </c>
+      <c r="R89" s="14" t="s">
+        <v>207</v>
+      </c>
       <c r="S89" s="55"/>
       <c r="T89" s="55"/>
       <c r="U89" s="55"/>
-      <c r="V89" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">64 =&gt; , </v>
-      </c>
+      <c r="V89" s="2"/>
       <c r="W89" s="55"/>
       <c r="X89" s="55"/>
       <c r="Z89" s="61"/>
@@ -5738,7 +6427,7 @@
     </row>
     <row r="90" spans="1:27" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B90" s="55" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C90" s="55"/>
       <c r="D90" s="55">
@@ -5752,12 +6441,12 @@
       </c>
       <c r="G90" s="55"/>
       <c r="H90" s="56">
-        <f t="shared" si="31"/>
+        <f t="shared" si="51"/>
         <v>128</v>
       </c>
       <c r="I90" s="55"/>
       <c r="J90" s="55" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="52"/>
         <v>80</v>
       </c>
       <c r="K90" s="55"/>
@@ -5765,20 +6454,23 @@
         <v>16</v>
       </c>
       <c r="M90" s="54" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="N90" s="55"/>
       <c r="O90" s="58"/>
-      <c r="P90" s="58"/>
-      <c r="Q90" s="58"/>
-      <c r="R90" s="55"/>
+      <c r="P90" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q90" s="3">
+        <v>0</v>
+      </c>
+      <c r="R90" s="14" t="s">
+        <v>203</v>
+      </c>
       <c r="S90" s="55"/>
       <c r="T90" s="55"/>
       <c r="U90" s="55"/>
-      <c r="V90" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">128 =&gt; , </v>
-      </c>
+      <c r="V90" s="2"/>
       <c r="W90" s="55"/>
       <c r="X90" s="55"/>
       <c r="Z90" s="61"/>
@@ -5786,7 +6478,7 @@
     </row>
     <row r="91" spans="1:27" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B91" s="55" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C91" s="55"/>
       <c r="D91" s="55">
@@ -5800,12 +6492,12 @@
       </c>
       <c r="G91" s="55"/>
       <c r="H91" s="56">
-        <f t="shared" si="31"/>
+        <f t="shared" si="51"/>
         <v>192</v>
       </c>
       <c r="I91" s="55"/>
       <c r="J91" s="55" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="52"/>
         <v>C0</v>
       </c>
       <c r="K91" s="55"/>
@@ -5813,17 +6505,20 @@
         <v>16</v>
       </c>
       <c r="M91" s="54" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N91" s="55"/>
       <c r="O91" s="58"/>
-      <c r="P91" s="58"/>
-      <c r="Q91" s="58"/>
-      <c r="R91" s="55"/>
-      <c r="V91" s="2" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">192 =&gt; , </v>
-      </c>
+      <c r="P91" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q91" s="3">
+        <v>0</v>
+      </c>
+      <c r="R91" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="V91" s="2"/>
       <c r="Z91" s="61"/>
       <c r="AA91" s="61"/>
     </row>
@@ -5844,7 +6539,7 @@
       <c r="Q92" s="64"/>
       <c r="R92" s="21"/>
       <c r="V92" s="73" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="Z92" s="16"/>
       <c r="AA92" s="65"/>

</xml_diff>